<commit_message>
docs(m3): evolve PED RTM registers and release evidence for review
</commit_message>
<xml_diff>
--- a/docs/CivicConnect_RTM_v2.0.xlsx
+++ b/docs/CivicConnect_RTM_v2.0.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" r:id="Rd7cc999ae4474c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R567844fcd7b94a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" r:id="R6efa84dfd90541a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Red4c5d83536246f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -72,6 +72,11 @@
         <x:fgColor rgb="FFF5F5F5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9D9D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -79,7 +84,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -116,6 +121,20 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -338,6 +357,10 @@
     <x:col min="18" max="18" width="48" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="32" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="32" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="65" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="65" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="65" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -395,6 +418,18 @@
       <x:c r="R1" s="11" t="str">
         <x:v>Current requirement wording</x:v>
       </x:c>
+      <x:c r="S1" s="20" t="str">
+        <x:v>Expected / observed result</x:v>
+      </x:c>
+      <x:c r="T1" s="20" t="str">
+        <x:v>Defect or remaining acceptance gap</x:v>
+      </x:c>
+      <x:c r="U1" s="20" t="str">
+        <x:v>M3 execution evidence</x:v>
+      </x:c>
+      <x:c r="V1" s="20" t="str">
+        <x:v>Evidence date / executor</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="95" customHeight="1">
       <x:c r="A2" s="3" t="str">
@@ -426,10 +461,10 @@
         <x:v>Creation and input validation not implemented</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L2" s="3" t="str">
         <x:v>Planned</x:v>
@@ -444,7 +479,7 @@
         <x:v>ServiceRequest, Category, RequestHistory; atomic creation and idempotency</x:v>
       </x:c>
       <x:c r="P2" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q2" s="14" t="str">
         <x:v>R-015; R-036</x:v>
@@ -453,6 +488,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A2,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow requesters to submit a request with a category, description and location.</x:v>
       </x:c>
+      <x:c r="S2" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T2" s="21" t="str">
+        <x:v>Request creation and input-validation endpoint absent.</x:v>
+      </x:c>
+      <x:c r="U2" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V2" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="95" customHeight="1">
       <x:c r="A3" s="6" t="str">
@@ -484,10 +531,10 @@
         <x:v>Controlled catalogue and persistent keys not implemented</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L3" s="6" t="str">
         <x:v>Planned</x:v>
@@ -502,7 +549,7 @@
         <x:v>Category FK; retain referenced category</x:v>
       </x:c>
       <x:c r="P3" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q3" s="15" t="str">
         <x:v>R-019</x:v>
@@ -511,6 +558,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A3,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Use a predefined list of request categories.</x:v>
       </x:c>
+      <x:c r="S3" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T3" s="21" t="str">
+        <x:v>Controlled category catalogue/enforced category key absent.</x:v>
+      </x:c>
+      <x:c r="U3" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V3" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="95" customHeight="1">
       <x:c r="A4" s="3" t="str">
@@ -536,16 +595,16 @@
         <x:v>ADR-M2-01; ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>Local: src/CivicConnect.Web/; tests/CivicConnect.Verification/Program.cs. Cameron M2 PR not created.</x:v>
+        <x:v>src/CivicConnect.Web/: RequestQueryService; RequestAccessPolicy; EfRequestReader; RequestStatusService. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>S01/S03; H04/H05/H07; initial read checks passed; docs/evidence/local-verification.txt</x:v>
+        <x:v>E01/E02/A04; S01/S03/H04/H05/H07; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K4" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L4" s="3" t="str">
         <x:v>In Development</x:v>
@@ -557,10 +616,10 @@
         <x:v>RequestsController; RequestQueryService</x:v>
       </x:c>
       <x:c r="O4" s="14" t="str">
-        <x:v>ServiceRequest ownership/status snapshot; PostgreSQL adapter planned</x:v>
+        <x:v>Michael EF Core/PostgreSQL reader and persisted synthetic requests/notes; authorised application projection.</x:v>
       </x:c>
       <x:c r="P4" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q4" s="14" t="str">
         <x:v>R-013; R-017</x:v>
@@ -569,6 +628,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A4,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow requesters to view the current status of their own requests.</x:v>
       </x:c>
+      <x:c r="S4" s="21" t="str">
+        <x:v>Owner reads saved Closed status/time and permitted notes; foreign record returns 404.</x:v>
+      </x:c>
+      <x:c r="T4" s="21" t="str">
+        <x:v>Full live account/UI acceptance pending. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U4" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V4" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="95" customHeight="1">
       <x:c r="A5" s="6" t="str">
@@ -600,10 +671,10 @@
         <x:v>List/history query not implemented</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K5" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L5" s="6" t="str">
         <x:v>Planned</x:v>
@@ -618,7 +689,7 @@
         <x:v>Requester-scoped ServiceRequest collection</x:v>
       </x:c>
       <x:c r="P5" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q5" s="15" t="str">
         <x:v>R-013</x:v>
@@ -627,6 +698,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A5,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow requesters to view their previous requests.</x:v>
       </x:c>
+      <x:c r="S5" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T5" s="21" t="str">
+        <x:v>Own request history/list workflow absent.</x:v>
+      </x:c>
+      <x:c r="U5" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V5" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="95" customHeight="1">
       <x:c r="A6" s="3" t="str">
@@ -652,19 +735,19 @@
         <x:v>ADR-M2-02; ADR-M2-03; ADR-M2-04; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
-        <x:v>Planned. Design source PR #10 (architecture) / #11 (data/technology); no application implementation for this row.</x:v>
+        <x:v>src/CivicConnect.Web/: RequestStatusService; EfRequestStatusWriter; EfRequestReader. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I6" s="3" t="str">
-        <x:v>Explicit coordination selected; no delivery implementation</x:v>
+        <x:v>E01/E02; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J6" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K6" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L6" s="3" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Development</x:v>
       </x:c>
       <x:c r="M6" s="14" t="str">
         <x:v>Integrity; access isolation</x:v>
@@ -673,10 +756,10 @@
         <x:v>Future change coordinator and feedback query</x:v>
       </x:c>
       <x:c r="O6" s="14" t="str">
-        <x:v>RequesterFeedback saved with required request/history changes</x:v>
+        <x:v>PostgreSQL status/history/public-note transaction and optimistic version; broader schema/acceptance gaps remain.</x:v>
       </x:c>
       <x:c r="P6" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q6" s="14" t="str">
         <x:v>R-027; R-028</x:v>
@@ -685,6 +768,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A6,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Provide requester feedback when a request is accepted, rejected, updated or completed.</x:v>
       </x:c>
+      <x:c r="S6" s="21" t="str">
+        <x:v>Status changes create persistent public feedback; rejection has a reason.</x:v>
+      </x:c>
+      <x:c r="T6" s="21" t="str">
+        <x:v>Event/date presentation and full feedback scope pending. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U6" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V6" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="95" customHeight="1">
       <x:c r="A7" s="6" t="str">
@@ -710,19 +805,19 @@
         <x:v>ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
-        <x:v>Planned. Design source PR #10 (architecture) / #11 (data/technology); no application implementation for this row.</x:v>
+        <x:v>src/CivicConnect.Web/: RequestAccessPolicy; request detail boundary only. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I7" s="6" t="str">
-        <x:v>Detail category policy exists; list acceptance not checked</x:v>
+        <x:v>S05/H09/BB05; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J7" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K7" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L7" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Development</x:v>
       </x:c>
       <x:c r="M7" s="15" t="str">
         <x:v>Access isolation</x:v>
@@ -734,7 +829,7 @@
         <x:v>Category permission filter before counts/pagination</x:v>
       </x:c>
       <x:c r="P7" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q7" s="15" t="str">
         <x:v>R-013; R-032</x:v>
@@ -743,6 +838,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A7,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow staff to view requests permitted by their role and assigned categories.</x:v>
       </x:c>
+      <x:c r="S7" s="21" t="str">
+        <x:v>Outside-category detail/mutation denied.</x:v>
+      </x:c>
+      <x:c r="T7" s="21" t="str">
+        <x:v>Authorised staff list absent. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U7" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V7" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="95" customHeight="1">
       <x:c r="A8" s="3" t="str">
@@ -774,10 +881,10 @@
         <x:v>No search, sorting or load evidence</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K8" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L8" s="3" t="str">
         <x:v>Planned</x:v>
@@ -792,7 +899,7 @@
         <x:v>Permission-constrained sort/filter/index strategy</x:v>
       </x:c>
       <x:c r="P8" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q8" s="14" t="str">
         <x:v>R-016; R-022</x:v>
@@ -801,6 +908,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A8,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow staff to search requests and filter by status, category, date and priority, and sort by date or priority.</x:v>
       </x:c>
+      <x:c r="S8" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T8" s="21" t="str">
+        <x:v>Search/filter/sort workflow absent.</x:v>
+      </x:c>
+      <x:c r="U8" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V8" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="95" customHeight="1">
       <x:c r="A9" s="6" t="str">
@@ -826,16 +945,16 @@
         <x:v>ADR-M2-01; ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
-        <x:v>Local: src/CivicConnect.Web/; tests/CivicConnect.Verification/Program.cs. Cameron M2 PR not created.</x:v>
+        <x:v>src/CivicConnect.Web/: RequestQueryService; RequestAccessPolicy; EfRequestReader. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I9" s="6" t="str">
-        <x:v>S04/S05; H08/H09; initial category/detail checks passed; docs/evidence/local-verification.txt</x:v>
+        <x:v>S04/S05/H08/H09; database checks; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J9" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K9" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L9" s="6" t="str">
         <x:v>In Development</x:v>
@@ -847,10 +966,10 @@
         <x:v>RequestsController; RequestQueryService</x:v>
       </x:c>
       <x:c r="O9" s="15" t="str">
-        <x:v>ServiceRequest and RequestNote read snapshot</x:v>
+        <x:v>Michael EF Core/PostgreSQL reader and persisted synthetic requests/notes; authorised application projection.</x:v>
       </x:c>
       <x:c r="P9" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q9" s="15" t="str">
         <x:v>R-013; R-017</x:v>
@@ -859,6 +978,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A9,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow authorised staff to view full request details.</x:v>
       </x:c>
+      <x:c r="S9" s="21" t="str">
+        <x:v>Permitted staff sees internal notes; wrong category denied.</x:v>
+      </x:c>
+      <x:c r="T9" s="21" t="str">
+        <x:v>Full details omit owner/priority/due-date/requester; AC1 incomplete. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U9" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V9" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="95" customHeight="1">
       <x:c r="A10" s="3" t="str">
@@ -890,10 +1021,10 @@
         <x:v>Database concurrency mechanism and simultaneous-claim test pending</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K10" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L10" s="3" t="str">
         <x:v>Planned</x:v>
@@ -908,7 +1039,7 @@
         <x:v>Conditional atomic owner update plus RequestHistory</x:v>
       </x:c>
       <x:c r="P10" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q10" s="14" t="str">
         <x:v>R-015</x:v>
@@ -917,6 +1048,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A10,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow authorised staff to assign a request or accept responsibility for it.</x:v>
       </x:c>
+      <x:c r="S10" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T10" s="21" t="str">
+        <x:v>Eligible owner assignment/concurrent claiming absent; Assigned status is not owner assignment.</x:v>
+      </x:c>
+      <x:c r="U10" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V10" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="95" customHeight="1">
       <x:c r="A11" s="6" t="str">
@@ -942,19 +1085,19 @@
         <x:v>ADR-M2-02; ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H11" s="6" t="str">
-        <x:v>Planned. Design source PR #10 (architecture) / #11 (data/technology); no application implementation for this row.</x:v>
+        <x:v>src/CivicConnect.Web/: StatusTransitionService; RequestStatusService; EfRequestStatusWriter. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I11" s="6" t="str">
-        <x:v>State code not present; no transition acceptance test</x:v>
+        <x:v>C01-C06; BB05; A03/A05/A06; E01/E02; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J11" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K11" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L11" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Development</x:v>
       </x:c>
       <x:c r="M11" s="15" t="str">
         <x:v>Integrity; testability</x:v>
@@ -963,10 +1106,10 @@
         <x:v>StatusTransitionService and State objects (planned)</x:v>
       </x:c>
       <x:c r="O11" s="15" t="str">
-        <x:v>State/history transaction; legal transition controlled by service</x:v>
+        <x:v>PostgreSQL status/history/public-note transaction and optimistic version; broader schema/acceptance gaps remain.</x:v>
       </x:c>
       <x:c r="P11" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q11" s="15" t="str">
         <x:v>R-011; R-027</x:v>
@@ -975,6 +1118,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A11,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow request status changes only through the agreed lifecycle.</x:v>
       </x:c>
+      <x:c r="S11" s="21" t="str">
+        <x:v>Legal lifecycle saved with actor/time/history; invalid/unauthorised/stale changes rejected.</x:v>
+      </x:c>
+      <x:c r="T11" s="21" t="str">
+        <x:v>Peer review/live identity and simultaneous HTTP/audit check pending. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U11" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V11" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="95" customHeight="1">
       <x:c r="A12" s="3" t="str">
@@ -1000,16 +1155,16 @@
         <x:v>ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
-        <x:v>Local: src/CivicConnect.Web/; tests/CivicConnect.Verification/Program.cs. Cameron M2 PR not created.</x:v>
+        <x:v>src/CivicConnect.Web/: DTO note filtering; EfRequestStatusWriter public feedback. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
-        <x:v>S02; H05/H08 protect read projection only; writes pending; docs/evidence/local-verification.txt</x:v>
+        <x:v>S02/H05; BB03/BB04; E01/E02; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K12" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L12" s="3" t="str">
         <x:v>In Development</x:v>
@@ -1021,10 +1176,10 @@
         <x:v>RequestQueryService note projection; note writing planned</x:v>
       </x:c>
       <x:c r="O12" s="14" t="str">
-        <x:v>RequestNote.IsRequesterVisible; author/history persistence planned</x:v>
+        <x:v>PostgreSQL status/history/public-note transaction and optimistic version; broader schema/acceptance gaps remain.</x:v>
       </x:c>
       <x:c r="P12" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q12" s="14" t="str">
         <x:v>R-017</x:v>
@@ -1033,6 +1188,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A12,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow staff to record comments, actions and resolution notes against a request.</x:v>
       </x:c>
+      <x:c r="S12" s="21" t="str">
+        <x:v>Internal notes excluded from owner response; invalid feedback produces no writes.</x:v>
+      </x:c>
+      <x:c r="T12" s="21" t="str">
+        <x:v>General note author/time/correction workflow absent. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U12" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V12" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="95" customHeight="1">
       <x:c r="A13" s="6" t="str">
@@ -1058,19 +1225,19 @@
         <x:v>ADR-M2-02; ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H13" s="6" t="str">
-        <x:v>Planned. Design source PR #10 (architecture) / #11 (data/technology); no application implementation for this row.</x:v>
+        <x:v>src/CivicConnect.Web/: StatusTransitionService; RequestStatusService; status POST. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I13" s="6" t="str">
-        <x:v>Resolve/close routes and tests pending</x:v>
+        <x:v>E01/E02; C01/C02; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J13" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K13" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L13" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Development</x:v>
       </x:c>
       <x:c r="M13" s="15" t="str">
         <x:v>Integrity; access isolation</x:v>
@@ -1079,10 +1246,10 @@
         <x:v>Resolution/closure use case (planned)</x:v>
       </x:c>
       <x:c r="O13" s="15" t="str">
-        <x:v>Status and required resolution note/history in transaction</x:v>
+        <x:v>PostgreSQL status/history/public-note transaction and optimistic version; broader schema/acceptance gaps remain.</x:v>
       </x:c>
       <x:c r="P13" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q13" s="15" t="str">
         <x:v>R-011; R-027</x:v>
@@ -1091,6 +1258,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A13,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow authorised staff to resolve and close requests.</x:v>
       </x:c>
+      <x:c r="S13" s="21" t="str">
+        <x:v>Staff resolves with summary then closes; terminal reopen denied.</x:v>
+      </x:c>
+      <x:c r="T13" s="21" t="str">
+        <x:v>Broader live account/permission acceptance pending. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U13" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V13" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="95" customHeight="1">
       <x:c r="A14" s="3" t="str">
@@ -1122,10 +1301,10 @@
         <x:v>No report implementation</x:v>
       </x:c>
       <x:c r="J14" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K14" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L14" s="3" t="str">
         <x:v>Planned</x:v>
@@ -1140,7 +1319,7 @@
         <x:v>Aggregate status/open/overdue queries</x:v>
       </x:c>
       <x:c r="P14" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q14" s="14" t="str">
         <x:v>R-014; R-016</x:v>
@@ -1149,6 +1328,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A14,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow management to view counts of open, overdue, resolved and closed requests.</x:v>
       </x:c>
+      <x:c r="S14" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T14" s="21" t="str">
+        <x:v>Management service counts absent.</x:v>
+      </x:c>
+      <x:c r="U14" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V14" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="95" customHeight="1">
       <x:c r="A15" s="6" t="str">
@@ -1180,10 +1371,10 @@
         <x:v>No grouping report implementation</x:v>
       </x:c>
       <x:c r="J15" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K15" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L15" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1198,7 +1389,7 @@
         <x:v>Aggregate Category/ServiceRequest grouping</x:v>
       </x:c>
       <x:c r="P15" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q15" s="15" t="str">
         <x:v>R-014; R-016</x:v>
@@ -1207,6 +1398,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A15,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow management to view requests and counts by category and status.</x:v>
       </x:c>
+      <x:c r="S15" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T15" s="21" t="str">
+        <x:v>Management category/status analysis absent.</x:v>
+      </x:c>
+      <x:c r="U15" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V15" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="95" customHeight="1">
       <x:c r="A16" s="3" t="str">
@@ -1232,19 +1435,19 @@
         <x:v>ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H16" s="3" t="str">
-        <x:v>Planned. Design source PR #10 (architecture) / #11 (data/technology); no application implementation for this row.</x:v>
+        <x:v>src/CivicConnect.Web/: RequestStatusHistoryEntity; EfRequestStatusWriter. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
-        <x:v>No durable history/report implementation</x:v>
+        <x:v>E01; database checks; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J16" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K16" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L16" s="3" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Development</x:v>
       </x:c>
       <x:c r="M16" s="14" t="str">
         <x:v>Integrity; access isolation</x:v>
@@ -1253,10 +1456,10 @@
         <x:v>Accountability reporting (planned)</x:v>
       </x:c>
       <x:c r="O16" s="14" t="str">
-        <x:v>Append-only RequestHistory actor/time/changes</x:v>
+        <x:v>PostgreSQL status/history/public-note transaction and optimistic version; broader schema/acceptance gaps remain.</x:v>
       </x:c>
       <x:c r="P16" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q16" s="14" t="str">
         <x:v>R-014</x:v>
@@ -1265,6 +1468,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A16,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Keep request history to support accountability and basic performance reporting.</x:v>
       </x:c>
+      <x:c r="S16" s="21" t="str">
+        <x:v>Four status audit edges with correct actor/time/version; history saved in PostgreSQL.</x:v>
+      </x:c>
+      <x:c r="T16" s="21" t="str">
+        <x:v>Creation/ownership/priority/due-date/note history and restart/immutability checks pending. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U16" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V16" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="95" customHeight="1">
       <x:c r="A17" s="6" t="str">
@@ -1290,16 +1505,16 @@
         <x:v>ADR-M2-01; ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H17" s="6" t="str">
-        <x:v>Local: src/CivicConnect.Web/; tests/CivicConnect.Verification/Program.cs. Cameron M2 PR not created.</x:v>
+        <x:v>src/CivicConnect.Web/: Cookie authentication; central action/read policy. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I17" s="6" t="str">
-        <x:v>S07-S12; H02/H03/H11; no real login or complete role routes; docs/evidence/local-verification.txt</x:v>
+        <x:v>A02/BB05; S07-S12/H02/H03; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J17" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K17" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L17" s="6" t="str">
         <x:v>In Development</x:v>
@@ -1314,7 +1529,7 @@
         <x:v>Trusted principal claims; user store/provisioning planned</x:v>
       </x:c>
       <x:c r="P17" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q17" s="15" t="str">
         <x:v>R-013; R-031; R-032</x:v>
@@ -1323,6 +1538,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A17,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Authenticate users and apply Requester, Staff and Management permissions.</x:v>
       </x:c>
+      <x:c r="S17" s="21" t="str">
+        <x:v>Signed-out calls return 401; ambiguous/inactive identities denied.</x:v>
+      </x:c>
+      <x:c r="T17" s="21" t="str">
+        <x:v>Actual credential login/provisioning and permission freshness absent. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U17" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V17" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="95" customHeight="1">
       <x:c r="A18" s="3" t="str">
@@ -1354,10 +1581,10 @@
         <x:v>No priority mutation implementation</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L18" s="3" t="str">
         <x:v>Planned</x:v>
@@ -1372,7 +1599,7 @@
         <x:v>Controlled Low/Normal/High; default Normal</x:v>
       </x:c>
       <x:c r="P18" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q18" s="14" t="str">
         <x:v>R-036</x:v>
@@ -1381,6 +1608,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A18,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Record a controlled priority for each request and allow authorised staff to change it.</x:v>
       </x:c>
+      <x:c r="S18" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T18" s="21" t="str">
+        <x:v>Controlled priority/default/update absent.</x:v>
+      </x:c>
+      <x:c r="U18" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V18" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="95" customHeight="1">
       <x:c r="A19" s="6" t="str">
@@ -1412,10 +1651,10 @@
         <x:v>No due-date/overdue implementation</x:v>
       </x:c>
       <x:c r="J19" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K19" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L19" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1430,7 +1669,7 @@
         <x:v>Open states plus DueDate &lt; now; null not overdue</x:v>
       </x:c>
       <x:c r="P19" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q19" s="15" t="str">
         <x:v>R-014</x:v>
@@ -1439,6 +1678,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A19,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow staff to record due dates and identify overdue requests.</x:v>
       </x:c>
+      <x:c r="S19" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T19" s="21" t="str">
+        <x:v>Due-date/overdue calculation absent.</x:v>
+      </x:c>
+      <x:c r="U19" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V19" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="95" customHeight="1">
       <x:c r="A20" s="3" t="str">
@@ -1464,16 +1715,16 @@
         <x:v>ADR-M2-01; ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H20" s="3" t="str">
-        <x:v>Local: src/CivicConnect.Web/; tests/CivicConnect.Verification/Program.cs. Cameron M2 PR not created.</x:v>
+        <x:v>src/CivicConnect.Web/: RequestAccessPolicy; filtered DTO; versioned status command. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
-        <x:v>S02-S12; H02-H09/H11; read subset only, no full access matrix pass; docs/evidence/local-verification.txt</x:v>
+        <x:v>C03/BB05/A04/A06/E01/E02; S02-S12; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J20" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K20" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L20" s="3" t="str">
         <x:v>In Development</x:v>
@@ -1485,10 +1736,10 @@
         <x:v>RequestAccessPolicy and DTO projection</x:v>
       </x:c>
       <x:c r="O20" s="14" t="str">
-        <x:v>Ownership/category/visibility; persistent permissions pending</x:v>
+        <x:v>Michael EF Core/PostgreSQL reader and persisted synthetic requests/notes; authorised application projection.</x:v>
       </x:c>
       <x:c r="P20" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q20" s="14" t="str">
         <x:v>R-013; R-017; R-032</x:v>
@@ -1497,6 +1748,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A20,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Protect requests using role and record-level access controls.</x:v>
       </x:c>
+      <x:c r="S20" s="21" t="str">
+        <x:v>No unauthorised disclosure/change in selected role/record cases.</x:v>
+      </x:c>
+      <x:c r="T20" s="21" t="str">
+        <x:v>Synthetic-ticket access matrix only; live permission freshness unverified. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U20" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V20" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="95" customHeight="1">
       <x:c r="A21" s="6" t="str">
@@ -1528,10 +1791,10 @@
         <x:v>Original load and timing targets unchanged; no measurements</x:v>
       </x:c>
       <x:c r="J21" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K21" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L21" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1546,7 +1809,7 @@
         <x:v>Indexes/pooling/data volume to verify</x:v>
       </x:c>
       <x:c r="P21" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q21" s="15" t="str">
         <x:v>R-016; R-022</x:v>
@@ -1555,6 +1818,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A21,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Complete at least 95% of submissions, status views, staff searches and management summaries within 3 seconds at pilot load, with at most 1% failures.</x:v>
       </x:c>
+      <x:c r="S21" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T21" s="21" t="str">
+        <x:v>No load measurements; original 3s/95%/1% target and pilot workload unverified.</x:v>
+      </x:c>
+      <x:c r="U21" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V21" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="95" customHeight="1">
       <x:c r="A22" s="3" t="str">
@@ -1580,19 +1855,19 @@
         <x:v>ADR-M2-02; ADR-M2-03; ADR-M2-04; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H22" s="3" t="str">
-        <x:v>Planned. Design source PR #10 (architecture) / #11 (data/technology); no application implementation for this row.</x:v>
+        <x:v>src/CivicConnect.Web/: EF transaction; concurrency version; status coordinator. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
-        <x:v>Fixture has no persistence; restart/double-click/rollback checks pending</x:v>
+        <x:v>A05/A06; E01; database checks; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J22" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K22" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L22" s="3" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Development</x:v>
       </x:c>
       <x:c r="M22" s="14" t="str">
         <x:v>Integrity</x:v>
@@ -1601,10 +1876,10 @@
         <x:v>Future transaction coordinator</x:v>
       </x:c>
       <x:c r="O22" s="14" t="str">
-        <x:v>Request/history/feedback atomicity; concurrency and idempotency</x:v>
+        <x:v>PostgreSQL status/history/public-note transaction and optimistic version; broader schema/acceptance gaps remain.</x:v>
       </x:c>
       <x:c r="P22" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q22" s="14" t="str">
         <x:v>R-015</x:v>
@@ -1613,6 +1888,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A22,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Save request data and its history together without partial updates.</x:v>
       </x:c>
+      <x:c r="S22" s="21" t="str">
+        <x:v>Failed status write rolls back; stale version rejected; saved effects agree.</x:v>
+      </x:c>
+      <x:c r="T22" s="21" t="str">
+        <x:v>Submission/assignment/idempotency and complete process restart unverified. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U22" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V22" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="95" customHeight="1">
       <x:c r="A23" s="6" t="str">
@@ -1644,10 +1931,10 @@
         <x:v>No representative participant evaluation</x:v>
       </x:c>
       <x:c r="J23" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K23" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L23" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1662,7 +1949,7 @@
         <x:v>No additional data decision</x:v>
       </x:c>
       <x:c r="P23" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q23" s="15" t="str">
         <x:v>R-021</x:v>
@@ -1671,6 +1958,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A23,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Make request submission and status checking easy for users with basic digital skills.</x:v>
       </x:c>
+      <x:c r="S23" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T23" s="21" t="str">
+        <x:v>No five-participant usability exercise.</x:v>
+      </x:c>
+      <x:c r="U23" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V23" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="95" customHeight="1">
       <x:c r="A24" s="3" t="str">
@@ -1702,10 +2001,10 @@
         <x:v>Landing exists; viewport/keyboard/core-route acceptance pending</x:v>
       </x:c>
       <x:c r="J24" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K24" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L24" s="3" t="str">
         <x:v>Planned</x:v>
@@ -1720,7 +2019,7 @@
         <x:v>No additional data decision</x:v>
       </x:c>
       <x:c r="P24" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q24" s="14" t="str">
         <x:v>R-021</x:v>
@@ -1729,6 +2028,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A24,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Provide a responsive web interface that supports keyboard use.</x:v>
       </x:c>
+      <x:c r="S24" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T24" s="21" t="str">
+        <x:v>No representative responsive/keyboard workflow evaluation.</x:v>
+      </x:c>
+      <x:c r="U24" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V24" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="95" customHeight="1">
       <x:c r="A25" s="6" t="str">
@@ -1754,19 +2065,19 @@
         <x:v>ADR-M2-01; ADR-M2-03; ADR-M2-04; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H25" s="6" t="str">
-        <x:v>Planned. Design source PR #10 (architecture) / #11 (data/technology); no application implementation for this row.</x:v>
+        <x:v>src/CivicConnect.Web/: Secure cookies; temporary HTTPS test host. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I25" s="6" t="str">
-        <x:v>Loopback HTTP tests do not validate deployed TLS</x:v>
+        <x:v>M3 suite ran over HTTPS; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J25" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K25" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L25" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Development</x:v>
       </x:c>
       <x:c r="M25" s="15" t="str">
         <x:v>Secure deployment constraint</x:v>
@@ -1778,7 +2089,7 @@
         <x:v>TLS for protected HTTP and database traffic</x:v>
       </x:c>
       <x:c r="P25" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q25" s="15" t="str">
         <x:v>R-033</x:v>
@@ -1787,6 +2098,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A25,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Use HTTPS to protect authentication and request data in deployed environments.</x:v>
       </x:c>
+      <x:c r="S25" s="21" t="str">
+        <x:v>Temporary loopback certificate and secure cookies used for test host.</x:v>
+      </x:c>
+      <x:c r="T25" s="21" t="str">
+        <x:v>Real deployed certificate/HTTPS redirect and browser acceptance pending. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U25" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V25" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="95" customHeight="1">
       <x:c r="A26" s="3" t="str">
@@ -1818,10 +2141,10 @@
         <x:v>RPO/RTO targets retained; no restore evidence</x:v>
       </x:c>
       <x:c r="J26" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K26" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L26" s="3" t="str">
         <x:v>Planned</x:v>
@@ -1836,7 +2159,7 @@
         <x:v>PostgreSQL backup and timed restore</x:v>
       </x:c>
       <x:c r="P26" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q26" s="14" t="str">
         <x:v>R-018; R-040</x:v>
@@ -1845,6 +2168,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A26,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Support recovery with no more than 24 hours of lost data and restoration within four hours.</x:v>
       </x:c>
+      <x:c r="S26" s="21" t="str">
+        <x:v>Not executed for complete acceptance.</x:v>
+      </x:c>
+      <x:c r="T26" s="21" t="str">
+        <x:v>No backup/restore measurement against RPO/RTO.</x:v>
+      </x:c>
+      <x:c r="U26" s="21" t="str">
+        <x:v>No complete M3 execution evidence; see docs/release-evidence.md.</x:v>
+      </x:c>
+      <x:c r="V26" s="21" t="str">
+        <x:v>2026-10-13 evidence review.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="95" customHeight="1">
       <x:c r="A27" s="6" t="str">
@@ -1870,16 +2205,16 @@
         <x:v>ADR-M2-01; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H27" s="6" t="str">
-        <x:v>Local: src/CivicConnect.Web/; tests/CivicConnect.Verification/Program.cs. Cameron M2 PR not created.</x:v>
+        <x:v>src/CivicConnect.Web/: Generic HTTP exception boundary. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I27" s="6" t="str">
-        <x:v>H05/H12/H13 passed; production log/secrets audit pending; docs/evidence/local-verification.txt</x:v>
+        <x:v>A05; H12/H13; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J27" s="6" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K27" s="6" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L27" s="6" t="str">
         <x:v>In Development</x:v>
@@ -1894,7 +2229,7 @@
         <x:v>Filtered DTO; generic exception handling</x:v>
       </x:c>
       <x:c r="P27" s="15" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q27" s="15" t="str">
         <x:v>R-034; R-035</x:v>
@@ -1903,6 +2238,18 @@
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A27,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Keep sensitive information out of application logs and error messages.</x:v>
       </x:c>
+      <x:c r="S27" s="21" t="str">
+        <x:v>500 does not disclose exception/private marker; responses no-store.</x:v>
+      </x:c>
+      <x:c r="T27" s="21" t="str">
+        <x:v>Full dummy-secret/log-content audit pending. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U27" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V27" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="95" customHeight="1">
       <x:c r="A28" s="3" t="str">
@@ -1928,16 +2275,16 @@
         <x:v>ADR-M2-01; ADR-M2-04; ADR-M2-05; ADR-M2-06; ADR-M2-07; docs/decisions/README.md</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>Local: src/CivicConnect.Web/; tests/CivicConnect.Verification/Program.cs. Cameron M2 PR not created.</x:v>
+        <x:v>src/CivicConnect.Web/: Injected reader/policy/writer; isolated executable suites. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>29 local checks passed; remaining core rules not implemented; docs/evidence/local-verification.txt</x:v>
+        <x:v>C01-C06; BB01-BB05; A01-A06; E01/E02; passed 2026-10-13 where mapped; docs/testing-m3.md.</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
-        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged</x:v>
+        <x:v>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</x:v>
       </x:c>
       <x:c r="K28" s="3" t="str">
-        <x:v>No release evidence</x:v>
+        <x:v>Local review baseline; release NOT READY; docs/release-evidence.md.</x:v>
       </x:c>
       <x:c r="L28" s="3" t="str">
         <x:v>In Development</x:v>
@@ -1952,7 +2299,7 @@
         <x:v>Synthetic data with controlled store fault</x:v>
       </x:c>
       <x:c r="P28" s="14" t="str">
-        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/PostgreSQL selected, adapter not built</x:v>
+        <x:v>ADR-M2-04: ASP.NET Core MVC/Razor; EF Core/Npgsql 8.0.11; PostgreSQL adapters/migrations implemented by Michael (PR14).</x:v>
       </x:c>
       <x:c r="Q28" s="14" t="str">
         <x:v>R-009; R-038</x:v>
@@ -1960,6 +2307,18 @@
       <x:c r="R28" s="14" t="str">
         <x:f>INDEX(Requirements!$B$2:$B$28,MATCH(A28,Requirements!$A$2:$A$28,0))</x:f>
         <x:v>Allow core request rules to be tested with controlled data in a separate test environment.</x:v>
+      </x:c>
+      <x:c r="S28" s="21" t="str">
+        <x:v>Repeatable core access/status cases; negative control fails forbidden transition.</x:v>
+      </x:c>
+      <x:c r="T28" s="21" t="str">
+        <x:v>Submission/assignment/reporting rules remain unimplemented. See docs/defects.md and technical-debt.md.</x:v>
+      </x:c>
+      <x:c r="U28" s="21" t="str">
+        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
+      </x:c>
+      <x:c r="V28" s="21" t="str">
+        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="45" customHeight="1">

</xml_diff>

<commit_message>
docs(m3): align final PED and RTM with personal verification
</commit_message>
<xml_diff>
--- a/docs/CivicConnect_RTM_v2.0.xlsx
+++ b/docs/CivicConnect_RTM_v2.0.xlsx
@@ -634,11 +634,15 @@
       <x:c r="T4" s="21" t="str">
         <x:v>Full live account/UI acceptance pending. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U4" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V4" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U4" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V4" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="5" ht="95" customHeight="1">
@@ -774,11 +778,15 @@
       <x:c r="T6" s="21" t="str">
         <x:v>Event/date presentation and full feedback scope pending. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U6" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V6" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U6" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V6" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7" ht="95" customHeight="1">
@@ -844,11 +852,15 @@
       <x:c r="T7" s="21" t="str">
         <x:v>Authorised staff list absent. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U7" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V7" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U7" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V7" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8" ht="95" customHeight="1">
@@ -984,11 +996,15 @@
       <x:c r="T9" s="21" t="str">
         <x:v>Full details omit owner/priority/due-date/requester; AC1 incomplete. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U9" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V9" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U9" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V9" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="10" ht="95" customHeight="1">
@@ -1124,11 +1140,15 @@
       <x:c r="T11" s="21" t="str">
         <x:v>Peer review/live identity and simultaneous HTTP/audit check pending. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U11" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V11" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U11" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V11" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="12" ht="95" customHeight="1">
@@ -1194,11 +1214,15 @@
       <x:c r="T12" s="21" t="str">
         <x:v>General note author/time/correction workflow absent. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U12" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V12" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U12" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V12" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="13" ht="95" customHeight="1">
@@ -1264,11 +1288,15 @@
       <x:c r="T13" s="21" t="str">
         <x:v>Broader live account/permission acceptance pending. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U13" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V13" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U13" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V13" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="14" ht="95" customHeight="1">
@@ -1474,11 +1502,15 @@
       <x:c r="T16" s="21" t="str">
         <x:v>Creation/ownership/priority/due-date/note history and restart/immutability checks pending. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U16" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V16" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U16" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V16" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="17" ht="95" customHeight="1">
@@ -1544,11 +1576,15 @@
       <x:c r="T17" s="21" t="str">
         <x:v>Actual credential login/provisioning and permission freshness absent. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U17" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V17" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U17" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V17" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="18" ht="95" customHeight="1">
@@ -1754,11 +1790,15 @@
       <x:c r="T20" s="21" t="str">
         <x:v>Synthetic-ticket access matrix only; live permission freshness unverified. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U20" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V20" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U20" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V20" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="21" ht="95" customHeight="1">
@@ -1894,11 +1934,15 @@
       <x:c r="T22" s="21" t="str">
         <x:v>Submission/assignment/idempotency and complete process restart unverified. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U22" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V22" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U22" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V22" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="23" ht="95" customHeight="1">
@@ -2104,11 +2148,15 @@
       <x:c r="T25" s="21" t="str">
         <x:v>Real deployed certificate/HTTPS redirect and browser acceptance pending. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U25" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V25" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U25" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V25" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="26" ht="95" customHeight="1">
@@ -2244,11 +2292,15 @@
       <x:c r="T27" s="21" t="str">
         <x:v>Full dummy-secret/log-content audit pending. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U27" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V27" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U27" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V27" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="28" ht="95" customHeight="1">
@@ -2314,11 +2366,15 @@
       <x:c r="T28" s="21" t="str">
         <x:v>Submission/assignment/reporting rules remain unimplemented. See docs/defects.md and technical-debt.md.</x:v>
       </x:c>
-      <x:c r="U28" s="21" t="str">
-        <x:v>docs/testing-m3.md; docs/evidence/m3/integration.txt, regression.txt, database.txt (specific IDs in column I).</x:v>
-      </x:c>
-      <x:c r="V28" s="21" t="str">
-        <x:v>2026-10-13; Codex executed; human review pending.</x:v>
+      <x:c r="U28" s="21" t="inlineStr">
+        <x:is>
+          <x:t>docs/testing-m3.md; docs/evidence/m3/personal-20261013-181846/ (integration.txt, regression.txt, database.txt; mapped IDs in column I).</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V28" s="21" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-13 18:18-18:19 SAST; Cameron Purdon 601963; f774bf8.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="31" ht="45" customHeight="1">

</xml_diff>

<commit_message>
docs(m3): preserve final team PED and RTM for publication review
</commit_message>
<xml_diff>
--- a/docs/CivicConnect_RTM_v2.0.xlsx
+++ b/docs/CivicConnect_RTM_v2.0.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30606"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_BA9878C59281B343BAF2F7B7C8F16ABD1338820B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\uni\year 3\SEN\Milestone 3\To be sub\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D0BAA35-3E44-4E53-AAE5-796FE33F0C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8595" yWindow="1605" windowWidth="29730" windowHeight="19080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RTM" sheetId="1" r:id="rId1"/>
@@ -32,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="457">
   <si>
     <t>Requirement ID</t>
   </si>
@@ -127,9 +132,6 @@
     <t>M2 consolidation 2026-09-30; requirement/AC unchanged; M3 2026-10-13: evidence evolved; requirement/AC unchanged; CR-M3-C01.</t>
   </si>
   <si>
-    <t>Local review baseline; release NOT READY; docs/release-evidence.md.</t>
-  </si>
-  <si>
     <t>Planned</t>
   </si>
   <si>
@@ -211,9 +213,6 @@
     <t>ADR-M2-01; ADR-M2-03; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: RequestQueryService; RequestAccessPolicy; EfRequestReader; RequestStatusService. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>E01/E02/A04; S01/S03/H04/H05/H07; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -292,18 +291,12 @@
     <t>ADR-M2-02; ADR-M2-03; ADR-M2-04; ADR-M2-06; docs/decisions/README.md</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: RequestStatusService; EfRequestStatusWriter; EfRequestReader. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>E01/E02; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
     <t>Integrity; access isolation</t>
   </si>
   <si>
-    <t>Future change coordinator and feedback query</t>
-  </si>
-  <si>
     <t>PostgreSQL status/history/public-note transaction and optimistic version; broader schema/acceptance gaps remain.</t>
   </si>
   <si>
@@ -331,9 +324,6 @@
     <t>AC-FR-006-1; AC-FR-006-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: RequestAccessPolicy; request detail boundary only. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>S05/H09/BB05; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -397,9 +387,6 @@
     <t>AC-FR-008-1; AC-FR-008-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: RequestQueryService; RequestAccessPolicy; EfRequestReader. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>S04/S05/H08/H09; database checks; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -451,21 +438,12 @@
     <t>AC-FR-010-1; AC-FR-010-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: StatusTransitionService; RequestStatusService; EfRequestStatusWriter. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>C01-C06; BB05; A03/A05/A06; E01/E02; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
     <t>Integrity; testability</t>
   </si>
   <si>
-    <t>StatusTransitionService and State objects (planned)</t>
-  </si>
-  <si>
-    <t>R-011; R-027</t>
-  </si>
-  <si>
     <t>Legal lifecycle saved with actor/time/history; invalid/unauthorised/stale changes rejected.</t>
   </si>
   <si>
@@ -484,18 +462,12 @@
     <t>AC-FR-011-1; AC-FR-011-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: DTO note filtering; EfRequestStatusWriter public feedback. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>S02/H05; BB03/BB04; E01/E02; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
     <t>Access isolation; integrity</t>
   </si>
   <si>
-    <t>RequestQueryService note projection; note writing planned</t>
-  </si>
-  <si>
     <t>R-017</t>
   </si>
   <si>
@@ -517,15 +489,9 @@
     <t>AC-FR-012-1; AC-FR-012-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: StatusTransitionService; RequestStatusService; status POST. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>E01/E02; C01/C02; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
-    <t>Resolution/closure use case (planned)</t>
-  </si>
-  <si>
     <t>Staff resolves with summary then closes; terminal reopen denied.</t>
   </si>
   <si>
@@ -604,9 +570,6 @@
     <t>AC-FR-015-1; AC-FR-015-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: RequestStatusHistoryEntity; EfRequestStatusWriter. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>E01; database checks; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -637,9 +600,6 @@
     <t>AC-FR-016-1; AC-FR-016-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: Cookie authentication; central action/read policy. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>A02/BB05; S07-S12/H02/H03; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -730,9 +690,6 @@
     <t>AC-NFR-001-1; AC-NFR-001-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: RequestAccessPolicy; filtered DTO; versioned status command. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>C03/BB05/A04/A06/E01/E02; S02-S12; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -766,21 +723,9 @@
     <t>ADR-M2-01; ADR-M2-03; ADR-M2-04; docs/decisions/README.md</t>
   </si>
   <si>
-    <t>Original load and timing targets unchanged; no measurements</t>
-  </si>
-  <si>
     <t>Pilot performance</t>
   </si>
   <si>
-    <t>Single application; later load harness</t>
-  </si>
-  <si>
-    <t>Indexes/pooling/data volume to verify</t>
-  </si>
-  <si>
-    <t>No load measurements; original 3s/95%/1% target and pilot workload unverified.</t>
-  </si>
-  <si>
     <t>NFR-003</t>
   </si>
   <si>
@@ -796,15 +741,9 @@
     <t>AC-NFR-003-1; AC-NFR-003-2</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: EF transaction; concurrency version; status coordinator. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>A05/A06; E01; database checks; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
-    <t>Future transaction coordinator</t>
-  </si>
-  <si>
     <t>Failed status write rolls back; stale version rejected; saved effects agree.</t>
   </si>
   <si>
@@ -892,9 +831,6 @@
     <t>ADR-M2-01; ADR-M2-03; ADR-M2-04; ADR-M2-06; docs/decisions/README.md</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: Secure cookies; temporary HTTPS test host. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>M3 suite ran over HTTPS; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -967,9 +903,6 @@
     <t>ADR-M2-01; ADR-M2-04; ADR-M2-05; ADR-M2-06; docs/decisions/README.md</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: Generic HTTP exception boundary. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>A05; H12/H13; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -1009,9 +942,6 @@
     <t>ADR-M2-01; ADR-M2-04; ADR-M2-05; ADR-M2-06; ADR-M2-07; docs/decisions/README.md</t>
   </si>
   <si>
-    <t>src/CivicConnect.Web/: Injected reader/policy/writer; isolated executable suites. M2 PR12; M3 PR14; local Cameron integration/test commit fef0469.</t>
-  </si>
-  <si>
     <t>C01-C06; BB01-BB05; A01-A06; E01/E02; passed 2026-10-13 where mapped; docs/testing-m3.md.</t>
   </si>
   <si>
@@ -1024,9 +954,6 @@
     <t>Synthetic data with controlled store fault</t>
   </si>
   <si>
-    <t>R-009; R-038</t>
-  </si>
-  <si>
     <t>Repeatable core access/status cases; negative control fails forbidden transition.</t>
   </si>
   <si>
@@ -1042,15 +969,9 @@
     <t>RTM format</t>
   </si>
   <si>
-    <t>M2 evolution: M1 requirements and ACs retained; M2 architecture/data/technology/design and local evidence added. Supporting research is in ADRs.</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Planned = no working implementation. In Development = partial local evidence; not full acceptance. No requirement marked Verified. Team baseline approval pending.</t>
-  </si>
-  <si>
     <t>Maintenance</t>
   </si>
   <si>
@@ -1379,6 +1300,114 @@
   </si>
   <si>
     <t>External messaging integrations, payments, multi-tenant support and native apps are excluded from the initial version. Attachments, automated escalation, public APIs, AI categorisation and multilingual support remain future scope. Technology and architecture decisions will be addressed in M2.</t>
+  </si>
+  <si>
+    <t>PERF-01: 200 reads, max 10 concurrent; 200 successes, 0 errors; 1.62 ms mean, 0.41 ms median, 8.69 ms p95; 0.12 s; 1696.16 ops/sec.</t>
+  </si>
+  <si>
+    <t>EfRequestReader; EF Core/PostgreSQL; separate concurrent-read benchmark</t>
+  </si>
+  <si>
+    <t>One temporary request; separate DbContext per read; setup/cleanup excluded from measured workload.</t>
+  </si>
+  <si>
+    <t>R-016; R-022; R-057; M3-R05</t>
+  </si>
+  <si>
+    <t>No separate database-level target. Observed: 200/200 reads succeed; 1.62 ms mean, 8.69 ms p95. Full user-visible pilot acceptance not established.</t>
+  </si>
+  <si>
+    <t>AC-NFR-002-1/2 unchanged: 1000 requests, 10 users, 10 minutes after 2-minute warm-up; user-visible timings/cold start untested. Exact execution commit not recorded.</t>
+  </si>
+  <si>
+    <t>14 October 2026; Michael Ellis 600332; macOS; SDK 8.0.425; EF Core 8; PostgreSQL 17. Second run confirmed through Cameron.</t>
+  </si>
+  <si>
+    <t>Reviewed 14 Oct 2026; baseline 3760605 (local tag). NOT READY; PED Section 14; docs/release-evidence.md.</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: RequestQueryService; RequestAccessPolicy; EfRequestReader; RequestStatusService. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>M2 requirement/AC unchanged; CR-M3-C01, 13 Oct 2026. Combined conformance review completed 14 Oct 2026; baseline 3760605.</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: RequestStatusService; EfRequestStatusWriter; EfRequestReader. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>RequestStatusService; transactional public feedback; authorised feedback projection</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: RequestAccessPolicy; request detail boundary only. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: RequestQueryService; RequestAccessPolicy; EfRequestReader. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: StatusTransitionService; RequestStatusService; EfRequestStatusWriter. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>StatusTransitionService; six State classes; RequestStatusService</t>
+  </si>
+  <si>
+    <t>R-011; R-027; R-047 closed for tested lifecycle; TD-04 closed for reviewed architecture (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: DTO note filtering; EfRequestStatusWriter public feedback. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>RequestQueryService note projection; transactional status-related public-note writer; general note workflow unimplemented</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: StatusTransitionService; RequestStatusService; status POST. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>RequestStatusService; State rules for resolution and closure; transactional history/feedback writer</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: RequestStatusHistoryEntity; EfRequestStatusWriter. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: Cookie authentication; central action/read policy. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: RequestAccessPolicy; filtered DTO; versioned status command. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>PR16: original source 4a7cebe; current head 7f0417b. tests/CivicConnect.PerformanceTests/Program.cs; EfRequestReader/PostgreSQL. Reviewed combined baseline 3760605.</t>
+  </si>
+  <si>
+    <t>M2 acceptance criteria unchanged. PERF-01 second run confirmed 14 Oct 2026; completed combined review and PR16 CI linked. Full pilot acceptance unverified.</t>
+  </si>
+  <si>
+    <t>PERF-01: docs/evidence/m3-performance-results.txt and m3-performance-run-confirmation.md; execution SHA unconfirmed. PR16 CI, head 7f0417b: https://github.com/Michael-Ellis819/Virtual_Group_K_SEN381_Project/actions/runs/38577509314 (performance and dependency audits; not the combined M3 suite).</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: EF transaction; concurrency version; status coordinator. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>RequestStatusService; EfRequestStatusWriter; transaction and optimistic concurrency</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: Secure cookies; temporary HTTPS test host. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: Generic HTTP exception boundary. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>src/CivicConnect.Web/: Injected reader/policy/writer; isolated executable suites. M2 PR12; M3 PR14; reviewed combined baseline 3760605 (14 Oct 2026).</t>
+  </si>
+  <si>
+    <t>R-009; R-038; R-047 closed for tested lifecycle; R-053 open (combined CI coverage).</t>
+  </si>
+  <si>
+    <t>Personal run: docs/evidence/m3/personal-20261013-181846/; mapped IDs in I28. PR16 CI: https://github.com/Michael-Ellis819/Virtual_Group_K_SEN381_Project/actions/runs/38577509314 (legacy/database/performance and dependency audits). Cameron's 19 M3 cases verified locally; combined remote run not evidenced.</t>
+  </si>
+  <si>
+    <t>M1/M2 requirements and acceptance criteria retained. M3 implementation/test evidence and completed combined review (14 Oct 2026) added. Review: docs/reviews/Bianca_M3_Final_Review_Updated.docx; baseline 3760605, local tag m3-combined-review-20261014.</t>
+  </si>
+  <si>
+    <t>Planned = no working implementation. In Development = partial evidence; full acceptance unverified. Combined work reviewed by Bianca and Michael on 14 Oct 2026. Formal repository approvals/combined CI are assessed separately in PED Section 14.</t>
   </si>
 </sst>
 </file>
@@ -1394,21 +1423,25 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1702,7 +1735,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V38"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.625" customWidth="1"/>
     <col min="2" max="2" width="26.125" customWidth="1"/>
@@ -1821,1946 +1854,1870 @@
       <c r="J2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K2" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>37</v>
       </c>
       <c r="R2" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A2,Requirements!$A$2:$A$28,0))</f>
         <v>Allow requesters to submit a request with a category, description and location.</v>
       </c>
       <c r="S2" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="T2" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="T2" s="8" t="s">
+      <c r="U2" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="U2" s="8" t="s">
+      <c r="V2" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V2" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="95.1" customHeight="1">
       <c r="A3" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C3" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>44</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>45</v>
       </c>
       <c r="E3" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A3,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F3" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="10" t="s">
         <v>46</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>47</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J3" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K3" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="N3" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="O3" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="P3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q3" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="R3" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A3,Requirements!$A$2:$A$28,0))</f>
         <v>Use a predefined list of request categories.</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T3" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="U3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V3" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V3" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="95.1" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E4" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A4,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="J4" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="L4" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="M4" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="s">
+      <c r="N4" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="O4" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="P4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q4" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="R4" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A4,Requirements!$A$2:$A$28,0))</f>
         <v>Allow requesters to view the current status of their own requests.</v>
       </c>
       <c r="S4" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="T4" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="U4" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="T4" s="8" t="s">
+      <c r="V4" s="8" t="s">
         <v>67</v>
-      </c>
-      <c r="U4" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="V4" s="8" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="95.1" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>24</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E5" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A5,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K5" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N5" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q5" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="O5" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="P5" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q5" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="R5" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A5,Requirements!$A$2:$A$28,0))</f>
         <v>Allow requesters to view their previous requests.</v>
       </c>
       <c r="S5" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T5" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="U5" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V5" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V5" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:22" ht="95.1" customHeight="1">
       <c r="A6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="E6" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A6,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="J6" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="M6" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="N6" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="O6" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="P6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q6" s="5" t="s">
         <v>87</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="P6" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>91</v>
       </c>
       <c r="R6" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A6,Requirements!$A$2:$A$28,0))</f>
         <v>Provide requester feedback when a request is accepted, rejected, updated or completed.</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="T6" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="U6" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V6" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="95.1" customHeight="1">
       <c r="A7" s="10" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E7" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A7,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F7" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>428</v>
+      </c>
+      <c r="L7" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q7" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
-      </c>
-      <c r="L7" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="P7" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q7" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="R7" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A7,Requirements!$A$2:$A$28,0))</f>
         <v>Allow staff to view requests permitted by their role and assigned categories.</v>
       </c>
       <c r="S7" s="8" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="T7" s="8" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="U7" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V7" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="95.1" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="E8" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A8,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>28</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K8" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K8" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="P8" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="R8" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A8,Requirements!$A$2:$A$28,0))</f>
         <v>Allow staff to search requests and filter by status, category, date and priority, and sort by date or priority.</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T8" s="8" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="U8" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V8" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V8" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="95.1" customHeight="1">
       <c r="A9" s="10" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="E9" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A9,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>121</v>
+        <v>434</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L9" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="N9" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="O9" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="P9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q9" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="P9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q9" s="6" t="s">
-        <v>65</v>
       </c>
       <c r="R9" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A9,Requirements!$A$2:$A$28,0))</f>
         <v>Allow authorised staff to view full request details.</v>
       </c>
       <c r="S9" s="8" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="T9" s="8" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="U9" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V9" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="95.1" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="E10" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A10,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>28</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K10" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K10" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="R10" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A10,Requirements!$A$2:$A$28,0))</f>
         <v>Allow authorised staff to assign a request or accept responsibility for it.</v>
       </c>
       <c r="S10" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T10" s="8" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="U10" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V10" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V10" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="95.1" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="E11" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A11,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>139</v>
+        <v>435</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>142</v>
+        <v>436</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>143</v>
+        <v>437</v>
       </c>
       <c r="R11" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A11,Requirements!$A$2:$A$28,0))</f>
         <v>Allow request status changes only through the agreed lifecycle.</v>
       </c>
       <c r="S11" s="8" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="U11" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V11" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="95.1" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="E12" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A12,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>150</v>
+        <v>438</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K12" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>153</v>
+        <v>439</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="P12" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="R12" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A12,Requirements!$A$2:$A$28,0))</f>
         <v>Allow staff to record comments, actions and resolution notes against a request.</v>
       </c>
       <c r="S12" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="T12" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="U12" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V12" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="95.1" customHeight="1">
       <c r="A13" s="10" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E13" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A13,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>161</v>
+        <v>440</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>163</v>
+        <v>441</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>143</v>
+        <v>437</v>
       </c>
       <c r="R13" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A13,Requirements!$A$2:$A$28,0))</f>
         <v>Allow authorised staff to resolve and close requests.</v>
       </c>
       <c r="S13" s="8" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="T13" s="8" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="U13" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V13" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:22" ht="95.1" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="E14" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A14,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>28</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K14" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K14" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="P14" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="R14" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A14,Requirements!$A$2:$A$28,0))</f>
         <v>Allow management to view counts of open, overdue, resolved and closed requests.</v>
       </c>
       <c r="S14" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T14" s="8" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="U14" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V14" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V14" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:22" ht="95.1" customHeight="1">
       <c r="A15" s="10" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="E15" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A15,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="J15" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K15" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K15" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="P15" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="R15" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A15,Requirements!$A$2:$A$28,0))</f>
         <v>Allow management to view requests and counts by category and status.</v>
       </c>
       <c r="S15" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T15" s="8" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="U15" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V15" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V15" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:22" ht="95.1" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="E16" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A16,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>190</v>
+        <v>442</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>191</v>
+        <v>177</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K16" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="P16" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="R16" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A16,Requirements!$A$2:$A$28,0))</f>
         <v>Keep request history to support accountability and basic performance reporting.</v>
       </c>
       <c r="S16" s="8" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="T16" s="8" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="U16" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V16" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:22" ht="95.1" customHeight="1">
       <c r="A17" s="10" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="E17" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A17,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>201</v>
+        <v>443</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K17" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="P17" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="R17" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A17,Requirements!$A$2:$A$28,0))</f>
         <v>Authenticate users and apply Requester, Staff and Management permissions.</v>
       </c>
       <c r="S17" s="8" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="T17" s="8" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="U17" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V17" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:22" ht="95.1" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="E18" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A18,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>28</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K18" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K18" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="P18" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q18" s="5" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="R18" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A18,Requirements!$A$2:$A$28,0))</f>
         <v>Record a controlled priority for each request and allow authorised staff to change it.</v>
       </c>
       <c r="S18" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T18" s="8" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="U18" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V18" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V18" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:22" ht="95.1" customHeight="1">
       <c r="A19" s="10" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
       <c r="E19" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A19,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="J19" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K19" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K19" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L19" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="M19" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="M19" s="6" t="s">
-        <v>33</v>
-      </c>
       <c r="N19" s="6" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="R19" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A19,Requirements!$A$2:$A$28,0))</f>
         <v>Allow staff to record due dates and identify overdue requests.</v>
       </c>
       <c r="S19" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T19" s="8" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="U19" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V19" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V19" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:22" ht="95.1" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="E20" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A20,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>232</v>
+        <v>444</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K20" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M20" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="N20" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="O20" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="N20" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="O20" s="5" t="s">
-        <v>64</v>
-      </c>
       <c r="P20" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q20" s="5" t="s">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="R20" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A20,Requirements!$A$2:$A$28,0))</f>
         <v>Protect requests using role and record-level access controls.</v>
       </c>
       <c r="S20" s="8" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="T20" s="8" t="s">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="U20" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V20" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:22" ht="95.1" customHeight="1">
       <c r="A21" s="10" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="E21" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A21,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>243</v>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>PR16 source 4a7cebe; tests/CivicConnect.PerformanceTests/Program.cs; EfRequestReader/PostgreSQL. Combined locally with Cameron status/API increment.</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>PERF-01: 200 reads, max 10 concurrent; 200 successes, 0 errors; 1.62 ms mean, 0.41 ms median, 8.69 ms p95; 0.12 s; 1696.16 ops/sec.</t>
-        </is>
-      </c>
-      <c r="J21" s="10" t="inlineStr">
-        <is>
-          <t>M2 acceptance criteria retained. 14 October 2026: PERF-01 and Michael second-run confirmation added; limited performance evidence only.</t>
-        </is>
-      </c>
-      <c r="K21" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
-      </c>
-      <c r="L21" s="10" t="inlineStr">
-        <is>
-          <t>In Development</t>
-        </is>
+        <v>227</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>445</v>
+      </c>
+      <c r="I21" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="J21" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="K21" s="10" t="s">
+        <v>428</v>
+      </c>
+      <c r="L21" s="10" t="s">
+        <v>59</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="N21" s="6" t="inlineStr">
-        <is>
-          <t>EfRequestReader; EF Core/PostgreSQL; separate concurrent-read benchmark</t>
-        </is>
-      </c>
-      <c r="O21" s="6" t="inlineStr">
-        <is>
-          <t>One temporary request; separate DbContext per read; setup/cleanup excluded from measured workload.</t>
-        </is>
+        <v>228</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>423</v>
       </c>
       <c r="P21" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q21" s="6" t="inlineStr">
-        <is>
-          <t>R-016; R-022; R-057; M3-R05</t>
-        </is>
+        <v>35</v>
+      </c>
+      <c r="Q21" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="R21" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A21,Requirements!$A$2:$A$28,0))</f>
         <v>Complete at least 95% of submissions, status views, staff searches and management summaries within 3 seconds at pilot load, with at most 1% failures.</v>
       </c>
-      <c r="S21" s="8" t="inlineStr">
-        <is>
-          <t>No separate database-level target. Observed: 200/200 reads succeed; 1.62 ms mean, 8.69 ms p95. Full user-visible pilot acceptance not established.</t>
-        </is>
-      </c>
-      <c r="T21" s="8" t="inlineStr">
-        <is>
-          <t>AC-NFR-002-1/2 unchanged: 1000 requests, 10 users, 10 minutes after 2-minute warm-up; user-visible timings/cold start untested. Exact execution commit not recorded.</t>
-        </is>
-      </c>
-      <c r="U21" s="8" t="inlineStr">
-        <is>
-          <t>docs/evidence/m3-performance-results.txt; docs/evidence/m3-performance-run-confirmation.md; PED 7.3.7. PR16 source 4a7cebe; execution SHA unconfirmed.</t>
-        </is>
-      </c>
-      <c r="V21" s="8" t="inlineStr">
-        <is>
-          <t>14 October 2026; Michael Ellis 600332; macOS; SDK 8.0.425; EF Core 8; PostgreSQL 17. Second run confirmed through Cameron.</t>
-        </is>
+      <c r="S21" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="T21" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="U21" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="V21" s="8" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="22" spans="1:22" ht="95.1" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="E22" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A22,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>254</v>
+        <v>448</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>255</v>
+        <v>234</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K22" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N22" s="5" t="s">
-        <v>256</v>
+        <v>449</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="P22" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q22" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="R22" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A22,Requirements!$A$2:$A$28,0))</f>
         <v>Save request data and its history together without partial updates.</v>
       </c>
       <c r="S22" s="8" t="s">
-        <v>257</v>
+        <v>235</v>
       </c>
       <c r="T22" s="8" t="s">
-        <v>258</v>
+        <v>236</v>
       </c>
       <c r="U22" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V22" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:22" ht="95.1" customHeight="1">
       <c r="A23" s="10" t="s">
-        <v>259</v>
+        <v>237</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>260</v>
+        <v>238</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>261</v>
+        <v>239</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="E23" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A23,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>263</v>
+        <v>241</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
       <c r="H23" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>265</v>
+        <v>243</v>
       </c>
       <c r="J23" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K23" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K23" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L23" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>266</v>
+        <v>244</v>
       </c>
       <c r="N23" s="6" t="s">
-        <v>267</v>
+        <v>245</v>
       </c>
       <c r="O23" s="6" t="s">
-        <v>268</v>
+        <v>246</v>
       </c>
       <c r="P23" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q23" s="6" t="s">
-        <v>269</v>
+        <v>247</v>
       </c>
       <c r="R23" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A23,Requirements!$A$2:$A$28,0))</f>
         <v>Make request submission and status checking easy for users with basic digital skills.</v>
       </c>
       <c r="S23" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T23" s="8" t="s">
-        <v>270</v>
+        <v>248</v>
       </c>
       <c r="U23" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V23" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V23" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:22" ht="95.1" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>272</v>
+        <v>250</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>273</v>
+        <v>251</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="E24" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A24,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>28</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>276</v>
+        <v>254</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K24" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K24" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="N24" s="5" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="O24" s="5" t="s">
-        <v>268</v>
+        <v>246</v>
       </c>
       <c r="P24" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q24" s="5" t="s">
-        <v>269</v>
+        <v>247</v>
       </c>
       <c r="R24" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A24,Requirements!$A$2:$A$28,0))</f>
         <v>Provide a responsive web interface that supports keyboard use.</v>
       </c>
       <c r="S24" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T24" s="8" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="U24" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V24" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V24" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:22" ht="95.1" customHeight="1">
       <c r="A25" s="10" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
       <c r="E25" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A25,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>286</v>
+        <v>450</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>287</v>
+        <v>264</v>
       </c>
       <c r="J25" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K25" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K25" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L25" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="N25" s="6" t="s">
-        <v>289</v>
+        <v>266</v>
       </c>
       <c r="O25" s="6" t="s">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="P25" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q25" s="6" t="s">
-        <v>291</v>
+        <v>268</v>
       </c>
       <c r="R25" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A25,Requirements!$A$2:$A$28,0))</f>
         <v>Use HTTPS to protect authentication and request data in deployed environments.</v>
       </c>
       <c r="S25" s="8" t="s">
-        <v>292</v>
+        <v>269</v>
       </c>
       <c r="T25" s="8" t="s">
-        <v>293</v>
+        <v>270</v>
       </c>
       <c r="U25" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V25" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="95.1" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>294</v>
+        <v>271</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>295</v>
+        <v>272</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>297</v>
+        <v>274</v>
       </c>
       <c r="E26" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A26,Requirements!$A$2:$A$28,0))</f>
         <v>Medium</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>298</v>
+        <v>275</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>28</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>299</v>
+        <v>276</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K26" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+      <c r="K26" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>300</v>
+        <v>277</v>
       </c>
       <c r="N26" s="5" t="s">
-        <v>301</v>
+        <v>278</v>
       </c>
       <c r="O26" s="5" t="s">
-        <v>302</v>
+        <v>279</v>
       </c>
       <c r="P26" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q26" s="5" t="s">
-        <v>303</v>
+        <v>280</v>
       </c>
       <c r="R26" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A26,Requirements!$A$2:$A$28,0))</f>
         <v>Support recovery with no more than 24 hours of lost data and restoration within four hours.</v>
       </c>
       <c r="S26" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T26" s="8" t="s">
-        <v>304</v>
+        <v>281</v>
       </c>
       <c r="U26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V26" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="V26" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="95.1" customHeight="1">
       <c r="A27" s="10" t="s">
-        <v>305</v>
+        <v>282</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>306</v>
+        <v>283</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>307</v>
+        <v>284</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>308</v>
+        <v>285</v>
       </c>
       <c r="E27" s="10" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A27,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>309</v>
+        <v>286</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>310</v>
+        <v>287</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>311</v>
+        <v>451</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>312</v>
+        <v>288</v>
       </c>
       <c r="J27" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K27" s="10" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K27" s="10" t="s">
+        <v>428</v>
       </c>
       <c r="L27" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>313</v>
+        <v>289</v>
       </c>
       <c r="N27" s="6" t="s">
-        <v>314</v>
+        <v>290</v>
       </c>
       <c r="O27" s="6" t="s">
-        <v>315</v>
+        <v>291</v>
       </c>
       <c r="P27" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q27" s="6" t="s">
-        <v>316</v>
+        <v>292</v>
       </c>
       <c r="R27" s="6" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A27,Requirements!$A$2:$A$28,0))</f>
         <v>Keep sensitive information out of application logs and error messages.</v>
       </c>
       <c r="S27" s="8" t="s">
-        <v>317</v>
+        <v>293</v>
       </c>
       <c r="T27" s="8" t="s">
-        <v>318</v>
+        <v>294</v>
       </c>
       <c r="U27" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V27" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="95.1" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>319</v>
+        <v>295</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>320</v>
+        <v>296</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>321</v>
+        <v>297</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>322</v>
+        <v>298</v>
       </c>
       <c r="E28" s="1" t="str">
         <f>INDEX(Requirements!$C$2:$C$28,MATCH(A28,Requirements!$A$2:$A$28,0))</f>
         <v>High</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>323</v>
+        <v>299</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>324</v>
+        <v>300</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>325</v>
+        <v>452</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>326</v>
+        <v>301</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K28" s="1" t="inlineStr">
-        <is>
-          <t>Local combined candidate m3-combined-review-20261014; release NOT READY. docs/release-evidence.md.</t>
-        </is>
+        <v>430</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>428</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>327</v>
+        <v>302</v>
       </c>
       <c r="N28" s="5" t="s">
-        <v>328</v>
+        <v>303</v>
       </c>
       <c r="O28" s="5" t="s">
-        <v>329</v>
+        <v>304</v>
       </c>
       <c r="P28" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q28" s="5" t="s">
-        <v>330</v>
+        <v>453</v>
       </c>
       <c r="R28" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A28,Requirements!$A$2:$A$28,0))</f>
         <v>Allow core request rules to be tested with controlled data in a separate test environment.</v>
       </c>
       <c r="S28" s="8" t="s">
-        <v>331</v>
+        <v>305</v>
       </c>
       <c r="T28" s="8" t="s">
-        <v>332</v>
+        <v>306</v>
       </c>
       <c r="U28" s="8" t="s">
-        <v>68</v>
+        <v>454</v>
       </c>
       <c r="V28" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:22" ht="45" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>333</v>
+        <v>307</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>334</v>
+        <v>308</v>
       </c>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
@@ -3775,10 +3732,10 @@
     </row>
     <row r="32" spans="1:22" ht="45" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>335</v>
+        <v>309</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>336</v>
+        <v>455</v>
       </c>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
@@ -3793,10 +3750,10 @@
     </row>
     <row r="33" spans="1:12" ht="45" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>337</v>
+        <v>310</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>338</v>
+        <v>456</v>
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
@@ -3811,10 +3768,10 @@
     </row>
     <row r="34" spans="1:12" ht="45" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>339</v>
+        <v>311</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>340</v>
+        <v>312</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34" s="12"/>
@@ -3827,12 +3784,12 @@
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:12" ht="42.75">
       <c r="A35" t="s">
-        <v>341</v>
+        <v>313</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>342</v>
+        <v>314</v>
       </c>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
@@ -3845,12 +3802,12 @@
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
     </row>
-    <row r="36" spans="1:12">
+    <row r="36" spans="1:12" ht="42.75">
       <c r="A36" t="s">
-        <v>343</v>
+        <v>315</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>344</v>
+        <v>316</v>
       </c>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
@@ -3863,12 +3820,12 @@
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
     </row>
-    <row r="37" spans="1:12">
+    <row r="37" spans="1:12" ht="42.75">
       <c r="A37" t="s">
-        <v>345</v>
+        <v>317</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>346</v>
+        <v>318</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -3881,12 +3838,12 @@
       <c r="K37" s="4"/>
       <c r="L37" s="4"/>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:12" ht="57">
       <c r="A38" t="s">
-        <v>347</v>
+        <v>319</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>348</v>
+        <v>320</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
@@ -3918,7 +3875,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E37"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.625" customWidth="1"/>
     <col min="2" max="2" width="48.875" customWidth="1"/>
@@ -3928,7 +3885,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1">
       <c r="A1" s="9" t="s">
-        <v>349</v>
+        <v>321</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>1</v>
@@ -3937,10 +3894,10 @@
         <v>4</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>350</v>
+        <v>322</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>351</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="42" customHeight="1">
@@ -3948,466 +3905,466 @@
         <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>352</v>
+        <v>324</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>354</v>
+        <v>326</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>355</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="42" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>356</v>
+        <v>328</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>357</v>
+        <v>329</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>358</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="42" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>359</v>
+        <v>331</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>360</v>
+        <v>332</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>361</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="42" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>362</v>
+        <v>334</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>364</v>
+        <v>336</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>365</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="42" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>366</v>
+        <v>338</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>367</v>
+        <v>339</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>368</v>
+        <v>340</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="42" customHeight="1">
       <c r="A7" s="10" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>369</v>
+        <v>341</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>370</v>
+        <v>342</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>371</v>
+        <v>343</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="42" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>372</v>
+        <v>344</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>373</v>
+        <v>345</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>374</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="42" customHeight="1">
       <c r="A9" s="10" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>375</v>
+        <v>347</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>376</v>
+        <v>348</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>377</v>
+        <v>349</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="42" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>378</v>
+        <v>350</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>379</v>
+        <v>351</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>380</v>
+        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="42" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>381</v>
+        <v>353</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>382</v>
+        <v>354</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>383</v>
+        <v>355</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="42" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>384</v>
+        <v>356</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>385</v>
+        <v>357</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>386</v>
+        <v>358</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="42" customHeight="1">
       <c r="A13" s="10" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>387</v>
+        <v>359</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>388</v>
+        <v>360</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>389</v>
+        <v>361</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="42" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>390</v>
+        <v>362</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>391</v>
-      </c>
       <c r="E14" s="1" t="s">
-        <v>392</v>
+        <v>364</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="42" customHeight="1">
       <c r="A15" s="10" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>393</v>
+        <v>365</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>394</v>
+        <v>366</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>395</v>
+        <v>367</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="42" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>396</v>
+        <v>368</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>397</v>
+        <v>369</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>398</v>
+        <v>370</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="42" customHeight="1">
       <c r="A17" s="10" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>399</v>
+        <v>371</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>400</v>
+        <v>372</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>401</v>
+        <v>373</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="42" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>402</v>
+        <v>374</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>403</v>
+        <v>375</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>404</v>
+        <v>376</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="42" customHeight="1">
       <c r="A19" s="10" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>405</v>
+        <v>377</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>406</v>
+        <v>378</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>407</v>
+        <v>379</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="42" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>408</v>
+        <v>380</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>409</v>
+        <v>381</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>410</v>
+        <v>382</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="57" customHeight="1">
       <c r="A21" s="10" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>411</v>
+        <v>383</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>412</v>
+        <v>384</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>413</v>
+        <v>385</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="42" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>414</v>
+        <v>386</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>415</v>
+        <v>387</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>416</v>
+        <v>388</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="42" customHeight="1">
       <c r="A23" s="10" t="s">
-        <v>259</v>
+        <v>237</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>417</v>
+        <v>389</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>418</v>
+        <v>390</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>419</v>
+        <v>391</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="42" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>420</v>
+        <v>392</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>421</v>
+        <v>393</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>422</v>
+        <v>394</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="42" customHeight="1">
       <c r="A25" s="10" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>423</v>
+        <v>395</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>424</v>
+        <v>396</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>425</v>
+        <v>397</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="42" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>294</v>
+        <v>271</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>426</v>
+        <v>398</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>363</v>
+        <v>335</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>427</v>
+        <v>399</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>428</v>
+        <v>400</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="42" customHeight="1">
       <c r="A27" s="10" t="s">
-        <v>305</v>
+        <v>282</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>429</v>
+        <v>401</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>430</v>
+        <v>402</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>431</v>
+        <v>403</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="42" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>319</v>
+        <v>295</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>432</v>
+        <v>404</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>433</v>
+        <v>405</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>434</v>
+        <v>406</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="57.95" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>435</v>
+        <v>407</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>436</v>
+        <v>408</v>
       </c>
       <c r="C31" s="11"/>
       <c r="D31" s="11"/>
@@ -4415,10 +4372,10 @@
     </row>
     <row r="32" spans="1:5" ht="57.95" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>437</v>
+        <v>409</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>438</v>
+        <v>410</v>
       </c>
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
@@ -4426,10 +4383,10 @@
     </row>
     <row r="33" spans="1:5" ht="57.95" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>439</v>
+        <v>411</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>440</v>
+        <v>412</v>
       </c>
       <c r="C33" s="11"/>
       <c r="D33" s="11"/>
@@ -4437,10 +4394,10 @@
     </row>
     <row r="34" spans="1:5" ht="57.95" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>441</v>
+        <v>413</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>442</v>
+        <v>414</v>
       </c>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
@@ -4448,10 +4405,10 @@
     </row>
     <row r="35" spans="1:5" ht="57.95" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>443</v>
+        <v>415</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>444</v>
+        <v>416</v>
       </c>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
@@ -4459,10 +4416,10 @@
     </row>
     <row r="36" spans="1:5" ht="57.95" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>445</v>
+        <v>417</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>446</v>
+        <v>418</v>
       </c>
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
@@ -4470,10 +4427,10 @@
     </row>
     <row r="37" spans="1:5" ht="57.95" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>447</v>
+        <v>419</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>448</v>
+        <v>420</v>
       </c>
       <c r="C37" s="11"/>
       <c r="D37" s="11"/>

</xml_diff>

<commit_message>
Finalise M3 submission scope and evidence
</commit_message>
<xml_diff>
--- a/docs/CivicConnect_RTM_v2.0.xlsx
+++ b/docs/CivicConnect_RTM_v2.0.xlsx
@@ -1854,8 +1854,10 @@
       <c r="J2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>428</v>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L2" s="1" t="s">
         <v>31</v>
@@ -1924,8 +1926,10 @@
       <c r="J3" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K3" s="10" t="s">
-        <v>428</v>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L3" s="10" t="s">
         <v>31</v>
@@ -1985,17 +1989,23 @@
       <c r="G4" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>429</v>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: RequestQueryService; RequestAccessPolicy; EfRequestReader; RequestStatusService. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I4" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>428</v>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L4" s="1" t="s">
         <v>59</v>
@@ -2064,8 +2074,10 @@
       <c r="J5" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K5" s="10" t="s">
-        <v>428</v>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L5" s="10" t="s">
         <v>31</v>
@@ -2125,17 +2137,23 @@
       <c r="G6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>431</v>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: RequestStatusService; EfRequestStatusWriter; EfRequestReader. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I6" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>428</v>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L6" s="1" t="s">
         <v>59</v>
@@ -2195,17 +2213,23 @@
       <c r="G7" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="H7" s="10" t="s">
-        <v>433</v>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: RequestAccessPolicy; request detail boundary only. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I7" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="J7" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>428</v>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L7" s="10" t="s">
         <v>59</v>
@@ -2274,8 +2298,10 @@
       <c r="J8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>428</v>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L8" s="1" t="s">
         <v>31</v>
@@ -2335,17 +2361,23 @@
       <c r="G9" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="10" t="s">
-        <v>434</v>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: RequestQueryService; RequestAccessPolicy; EfRequestReader. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I9" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="J9" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>428</v>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L9" s="10" t="s">
         <v>59</v>
@@ -2414,8 +2446,10 @@
       <c r="J10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K10" s="1" t="s">
-        <v>428</v>
+      <c r="K10" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L10" s="1" t="s">
         <v>31</v>
@@ -2475,17 +2509,23 @@
       <c r="G11" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="H11" s="10" t="s">
-        <v>435</v>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: StatusTransitionService; RequestStatusService; EfRequestStatusWriter. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I11" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="J11" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="K11" s="10" t="s">
-        <v>428</v>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>Original requirement/AC unchanged. CR-M3-C03: team M3 scope confirmed 15 Oct; read/status increment conditionally ready in controlled simulation. PR17 and combined CI complete.</t>
+        </is>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L11" s="10" t="s">
         <v>59</v>
@@ -2512,8 +2552,10 @@
       <c r="S11" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="T11" s="8" t="s">
-        <v>136</v>
+      <c r="T11" s="8" t="inlineStr">
+        <is>
+          <t>Synthetic identities; simultaneous HTTP/audit coverage limited. Team accepts controlled M3 simulation; live accounts and full product remain incomplete for M4 finalisation.</t>
+        </is>
       </c>
       <c r="U11" s="8" t="s">
         <v>66</v>
@@ -2545,17 +2587,23 @@
       <c r="G12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>438</v>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: DTO note filtering; EfRequestStatusWriter public feedback. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I12" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>428</v>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L12" s="1" t="s">
         <v>59</v>
@@ -2615,17 +2663,23 @@
       <c r="G13" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="H13" s="10" t="s">
-        <v>440</v>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: StatusTransitionService; RequestStatusService; status POST. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I13" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="J13" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="K13" s="10" t="s">
-        <v>428</v>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L13" s="10" t="s">
         <v>59</v>
@@ -2694,8 +2748,10 @@
       <c r="J14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K14" s="1" t="s">
-        <v>428</v>
+      <c r="K14" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L14" s="1" t="s">
         <v>31</v>
@@ -2764,8 +2820,10 @@
       <c r="J15" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K15" s="10" t="s">
-        <v>428</v>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L15" s="10" t="s">
         <v>31</v>
@@ -2825,17 +2883,23 @@
       <c r="G16" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>442</v>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: RequestStatusHistoryEntity; EfRequestStatusWriter. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I16" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="J16" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>428</v>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K16" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L16" s="1" t="s">
         <v>59</v>
@@ -2895,17 +2959,23 @@
       <c r="G17" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="H17" s="10" t="s">
-        <v>443</v>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: Cookie authentication; central action/read policy. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I17" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="J17" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="K17" s="10" t="s">
-        <v>428</v>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L17" s="10" t="s">
         <v>59</v>
@@ -2974,8 +3044,10 @@
       <c r="J18" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K18" s="1" t="s">
-        <v>428</v>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L18" s="1" t="s">
         <v>31</v>
@@ -3044,8 +3116,10 @@
       <c r="J19" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K19" s="10" t="s">
-        <v>428</v>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L19" s="10" t="s">
         <v>31</v>
@@ -3105,17 +3179,23 @@
       <c r="G20" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>444</v>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: RequestAccessPolicy; filtered DTO; versioned status command. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I20" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>428</v>
+      <c r="J20" s="1" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K20" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L20" s="1" t="s">
         <v>59</v>
@@ -3175,17 +3255,23 @@
       <c r="G21" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="H21" s="10" t="s">
-        <v>445</v>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>tests/CivicConnect.PerformanceTests/Program.cs; EfRequestReader/PostgreSQL. PR16 performance merged into combined published implementation 668795a through PR17.</t>
+        </is>
       </c>
       <c r="I21" s="10" t="s">
         <v>421</v>
       </c>
-      <c r="J21" s="10" t="s">
-        <v>446</v>
-      </c>
-      <c r="K21" s="10" t="s">
-        <v>428</v>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>M2 acceptance criteria unchanged. Original PERF-01 second run confirmed 14 Oct; combined main CI passes on 668795a. Full pilot acceptance remains unverified.</t>
+        </is>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L21" s="10" t="s">
         <v>59</v>
@@ -3215,8 +3301,10 @@
       <c r="T21" s="8" t="s">
         <v>426</v>
       </c>
-      <c r="U21" s="8" t="s">
-        <v>447</v>
+      <c r="U21" s="8" t="inlineStr">
+        <is>
+          <t>PERF-01: docs/evidence/m3-performance-results.txt and m3-performance-run-confirmation.md; original execution SHA unconfirmed. Combined main CI on 668795a: https://github.com/Michael-Ellis819/Virtual_Group_K_SEN381_Project/actions/runs/38594557024 (all four projects; separate from original human benchmark).</t>
+        </is>
       </c>
       <c r="V21" s="8" t="s">
         <v>427</v>
@@ -3245,17 +3333,23 @@
       <c r="G22" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>448</v>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: EF transaction; concurrency version; status coordinator. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I22" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>428</v>
+      <c r="J22" s="1" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K22" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L22" s="1" t="s">
         <v>59</v>
@@ -3324,8 +3418,10 @@
       <c r="J23" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="K23" s="10" t="s">
-        <v>428</v>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L23" s="10" t="s">
         <v>31</v>
@@ -3394,8 +3490,10 @@
       <c r="J24" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K24" s="1" t="s">
-        <v>428</v>
+      <c r="K24" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L24" s="1" t="s">
         <v>31</v>
@@ -3455,17 +3553,23 @@
       <c r="G25" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="H25" s="10" t="s">
-        <v>450</v>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: Secure cookies; temporary HTTPS test host. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I25" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="J25" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="K25" s="10" t="s">
-        <v>428</v>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L25" s="10" t="s">
         <v>59</v>
@@ -3534,8 +3638,10 @@
       <c r="J26" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K26" s="1" t="s">
-        <v>428</v>
+      <c r="K26" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L26" s="1" t="s">
         <v>31</v>
@@ -3595,17 +3701,23 @@
       <c r="G27" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="H27" s="10" t="s">
-        <v>451</v>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: Generic HTTP exception boundary. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I27" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="J27" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="K27" s="10" t="s">
-        <v>428</v>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L27" s="10" t="s">
         <v>59</v>
@@ -3665,17 +3777,23 @@
       <c r="G28" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>452</v>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>src/CivicConnect.Web/: Injected reader/policy/writer; isolated executable suites. M2 PR12; M3 PR14; published combined implementation 668795a (PR17).</t>
+        </is>
       </c>
       <c r="I28" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="J28" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>428</v>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>M2 requirement/AC unchanged; CR-M3-C01 retained. Bianca/Michael review and PR17 approvals: 14 Oct. Published 668795a; CI verified; docs 15 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="inlineStr">
+        <is>
+          <t>15 Oct 2026; 668795a; PR17/CI pass. CONDITIONALLY READY: agreed M3 read/status increment, simulated staging only. PED Section 14.</t>
+        </is>
       </c>
       <c r="L28" s="1" t="s">
         <v>59</v>
@@ -3692,8 +3810,10 @@
       <c r="P28" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="Q28" s="5" t="s">
-        <v>453</v>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>R-009; R-038; R-047 closed for tested lifecycle; R-053 closed for current combined CI coverage (run 38594557024).</t>
+        </is>
       </c>
       <c r="R28" s="5" t="str">
         <f>INDEX(Requirements!$B$2:$B$28,MATCH(A28,Requirements!$A$2:$A$28,0))</f>
@@ -3702,11 +3822,15 @@
       <c r="S28" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="T28" s="8" t="s">
-        <v>306</v>
-      </c>
-      <c r="U28" s="8" t="s">
-        <v>454</v>
+      <c r="T28" s="8" t="inlineStr">
+        <is>
+          <t>Submission/assignment/reporting and real login remain original requirements planned for M4 finalisation; current evidence covers the agreed M3 read/status increment.</t>
+        </is>
+      </c>
+      <c r="U28" s="8" t="inlineStr">
+        <is>
+          <t>Personal run: docs/evidence/m3/personal-20261013-181846/; IDs in I28. Combined main CI: https://github.com/Michael-Ellis819/Virtual_Group_K_SEN381_Project/actions/runs/38594557024 on 668795a; regression/database/M3/performance, analysis and dependency checks pass.</t>
+        </is>
       </c>
       <c r="V28" s="8" t="s">
         <v>67</v>
@@ -3734,8 +3858,10 @@
       <c r="A32" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="B32" s="11" t="s">
-        <v>455</v>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Original requirements/ACs retained. Published 668795a; PR17 approvals and main CI 38594557024 pass. Cameron confirmed team M3 read/status scope on 15 Oct 2026. CONDITIONALLY READY for controlled simulated staging; CR-M3-C03 and PED Section 14.</t>
+        </is>
       </c>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
@@ -3752,8 +3878,10 @@
       <c r="A33" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="B33" s="11" t="s">
-        <v>456</v>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Planned = no working implementation. In Development = partial evidence; full acceptance unverified. Team plans unfinished original features for M4 finalisation; no requirements removed. M3 conditional readiness applies only to the agreed increment and simulation.</t>
+        </is>
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>

</xml_diff>

<commit_message>
Consolidate final M4 PED RTM and observed acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/CivicConnect_RTM_v2.0.xlsx
+++ b/docs/CivicConnect_RTM_v2.0.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" r:id="R9dc2dd3379a94e9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Rff3f11f5946f47f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" r:id="Rd8096fd30cef474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Rf8a8c07e99fc48c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1756,7 +1756,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="W1" s="16" t="str">
-        <x:v>M4 implementation checkpoint</x:v>
+        <x:v>M4 final implementation</x:v>
       </x:c>
       <x:c r="X1" s="16" t="str">
         <x:v>AC1 outcome</x:v>
@@ -1774,13 +1774,13 @@
         <x:v>Requirement value</x:v>
       </x:c>
       <x:c r="AC1" s="16" t="str">
-        <x:v>M4 evidence and scope</x:v>
+        <x:v>Final evidence</x:v>
       </x:c>
       <x:c r="AD1" s="16" t="str">
-        <x:v>Remaining integration / acceptance gap</x:v>
+        <x:v>Known limitation</x:v>
       </x:c>
       <x:c r="AE1" s="16" t="str">
-        <x:v>Checkpoint disposition</x:v>
+        <x:v>Final disposition</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="95.0999984741211" customHeight="1">
@@ -1855,34 +1855,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W2" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X2" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y2" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z2" s="17" t="n">
         <x:f>IF(X2="Met",1,IF(X2="Partially Met",0.5,IF(X2="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA2" s="17" t="n">
         <x:f>IF(Y2="Met",1,IF(Y2="Partially Met",0.5,IF(Y2="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB2" s="17" t="n">
         <x:f>IF(COUNT(Z2:AA2)=2,SUM(Z2:AA2),"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC2" s="15" t="str">
-        <x:v>Submission form and rejection boundaries tested; durable creation awaits the shared adapter. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P03–P06 exercise real submission, validation, reference/date/New/default priority, failed-write rollback and durable repeated submission. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD2" s="15" t="str">
-        <x:v>Valid submissions cannot yet be saved by the normal product.</x:v>
+        <x:v>Controlled synthetic records; no attachments or external notifications are in the baseline.</x:v>
       </x:c>
       <x:c r="AE2" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="95.0999984741211" customHeight="1">
@@ -1957,34 +1957,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W3" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X3" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y3" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z3" s="17" t="n">
         <x:f>IF(X3="Met",1,IF(X3="Partially Met",0.5,IF(X3="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA3" s="17" t="n">
         <x:f>IF(Y3="Met",1,IF(Y3="Partially Met",0.5,IF(Y3="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB3" s="17" t="n">
         <x:f>IF(COUNT(Z3:AA3)=2,SUM(Z3:AA3),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC3" s="15" t="str">
-        <x:v>Seven baseline categories offered; unlisted categories rejected by the controller. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P03/P05 save an agreed category and reject unlisted values; saved category is read back through the real reader. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD3" s="15" t="str">
-        <x:v>Catalogue persistence and retention must be verified with Michael’s adapter.</x:v>
+        <x:v>The seven-category catalogue is controlled in PortalOptions; a separate administrative category editor was not committed.</x:v>
       </x:c>
       <x:c r="AE3" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="95.0999984741211" customHeight="1">
@@ -2084,10 +2084,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AC4" s="15" t="str">
-        <x:v>M3 E01/E02/A04 verify saved own status/date and foreign denial; Razor details added. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P07/P24/P26 verify saved own status/date after updates and direct foreign denial; M3 E01/E02 remain regression evidence. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD4" s="15" t="str">
-        <x:v>Real account adapter is still absent; this trace covers controlled read/status behaviour.</x:v>
+        <x:v>Controlled accounts and local staging; no public production access is claimed.</x:v>
       </x:c>
       <x:c r="AE4" s="15" t="str">
         <x:v>Verified</x:v>
@@ -2165,34 +2165,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W5" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X5" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y5" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z5" s="17" t="n">
         <x:f>IF(X5="Met",1,IF(X5="Partially Met",0.5,IF(X5="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA5" s="17" t="n">
         <x:f>IF(Y5="Met",1,IF(Y5="Partially Met",0.5,IF(Y5="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB5" s="17" t="n">
         <x:f>IF(COUNT(Z5:AA5)=2,SUM(Z5:AA5),"Pending")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC5" s="15" t="str">
-        <x:v>Requester list view and ownership contract exercised with synthetic records. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P08/P26 show own saved reference/category/date/status, completed requests and foreign exclusion; UI checks cover the empty message. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD5" s="15" t="str">
-        <x:v>Persistent requester list and empty/history cases await integration.</x:v>
+        <x:v>Lists are unpaginated at the pilot scale.</x:v>
       </x:c>
       <x:c r="AE5" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="95.0999984741211" customHeight="1">
@@ -2292,10 +2292,10 @@
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="AC6" s="15" t="str">
-        <x:v>Status feedback persists; requester projection excludes internal notes. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P05/P12/P15/P24/P26 verify dated saved creation/assignment/status feedback and private-note exclusion. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD6" s="15" t="str">
-        <x:v>Dated feedback for every required event is not yet available in the product.</x:v>
+        <x:v>Status is shown in current details and dated status history. General public notes are not stored with their own separate status snapshot, so AC1 remains partial.</x:v>
       </x:c>
       <x:c r="AE6" s="15" t="str">
         <x:v>Not delivered</x:v>
@@ -2377,17 +2377,17 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="W7" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X7" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y7" s="15" t="str">
         <x:v>Met</x:v>
       </x:c>
       <x:c r="Z7" s="17" t="n">
         <x:f>IF(X7="Met",1,IF(X7="Partially Met",0.5,IF(X7="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA7" s="17" t="n">
         <x:f>IF(Y7="Met",1,IF(Y7="Partially Met",0.5,IF(Y7="Not Met",0,"Pending")))</x:f>
@@ -2395,16 +2395,16 @@
       </x:c>
       <x:c r="AB7" s="17" t="n">
         <x:f>IF(COUNT(Z7:AA7)=2,SUM(Z7:AA7),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC7" s="15" t="str">
-        <x:v>Staff list view prepared; M3 category/direct-access denial remains verified. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P07/P08 use real authorised/category-scoped queries and deny direct wrong-category detail access. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD7" s="15" t="str">
-        <x:v>The authorised persisted collection query is not implemented by this contribution.</x:v>
+        <x:v>Checks cover the supplied role/category dataset rather than an exhaustive penetration test.</x:v>
       </x:c>
       <x:c r="AE7" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="95.0999984741211" customHeight="1">
@@ -2479,34 +2479,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W8" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X8" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y8" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z8" s="17" t="n">
         <x:f>IF(X8="Met",1,IF(X8="Partially Met",0.5,IF(X8="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA8" s="17" t="n">
         <x:f>IF(Y8="Met",1,IF(Y8="Partially Met",0.5,IF(Y8="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB8" s="17" t="n">
         <x:f>IF(COUNT(Z8:AA8)=2,SUM(Z8:AA8),"Pending")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC8" s="15" t="str">
-        <x:v>Filter inputs, inclusive UTC dates and invalid ranges are checked. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P19/P20/P20a exercise combined authorised matching, exact UTC boundaries and Low/Normal/High sorting in both directions; clear/no-match rendering is covered by the UI suite. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD8" s="15" t="str">
-        <x:v>Actual matching, combined query results and priority/date ordering require the real data adapter.</x:v>
+        <x:v>No pagination or ranked full-text search is provided.</x:v>
       </x:c>
       <x:c r="AE8" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="95.0999984741211" customHeight="1">
@@ -2585,34 +2585,34 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="W9" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X9" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y9" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z9" s="17" t="n">
         <x:f>IF(X9="Met",1,IF(X9="Partially Met",0.5,IF(X9="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA9" s="17" t="n">
         <x:f>IF(Y9="Met",1,IF(Y9="Partially Met",0.5,IF(Y9="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB9" s="17" t="n">
         <x:f>IF(COUNT(Z9:AA9)=2,SUM(Z9:AA9),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC9" s="15" t="str">
-        <x:v>Protected details show the existing saved fields; extension fields render through the contract. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P07/P09 and the saved browser journey show all required detail fields, creation date, missing owner/due labels and access denial. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD9" s="15" t="str">
-        <x:v>Requester/owner/priority/due-date metadata is absent from current persistence.</x:v>
+        <x:v>Requesters receive a restricted projection; account IDs identify staff in the controlled demonstration.</x:v>
       </x:c>
       <x:c r="AE9" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="95.0999984741211" customHeight="1">
@@ -2687,34 +2687,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W10" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X10" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y10" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z10" s="17" t="n">
         <x:f>IF(X10="Met",1,IF(X10="Partially Met",0.5,IF(X10="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA10" s="17" t="n">
         <x:f>IF(Y10="Met",1,IF(Y10="Partially Met",0.5,IF(Y10="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB10" s="17" t="n">
         <x:f>IF(COUNT(Z10:AA10)=2,SUM(Z10:AA10),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC10" s="15" t="str">
-        <x:v>Bianca’s eligibility rule and Cameron’s assignment controller are tested in isolation. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P10/P10a/P11/P11a/P12 verify owner eligibility, actor/time, ownerless API rejection, rollback and two simultaneous HTTP claims yielding one saved owner. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD10" s="15" t="str">
-        <x:v>Atomic persisted ownership, audit and simultaneous claims remain unverified.</x:v>
+        <x:v>Concurrency was checked for the controlled two-claim race, not a production load profile.</x:v>
       </x:c>
       <x:c r="AE10" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="95.0999984741211" customHeight="1">
@@ -2816,10 +2816,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AC11" s="15" t="str">
-        <x:v>M3 C01–C06/A03/A05/A06/E01/E02 plus 36-pair LC matrix verify status legality and rejection. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>LC matrix, M3 C01/C02, P10b/P22/P24/P25 verify legal status/history writes and invalid, terminal and unauthorised rejection. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD11" s="15" t="str">
-        <x:v>Writer bypass remains debt; added entry points and final adapters require another integration run.</x:v>
+        <x:v>One source project still permits privileged code to reach EF directly; supported HTTP paths and writer boundaries are guarded.</x:v>
       </x:c>
       <x:c r="AE11" s="15" t="str">
         <x:v>Verified</x:v>
@@ -2901,34 +2901,34 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="W12" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X12" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y12" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z12" s="17" t="n">
         <x:f>IF(X12="Met",1,IF(X12="Partially Met",0.5,IF(X12="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA12" s="17" t="n">
         <x:f>IF(Y12="Met",1,IF(Y12="Partially Met",0.5,IF(Y12="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB12" s="17" t="n">
         <x:f>IF(COUNT(Z12:AA12)=2,SUM(Z12:AA12),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC12" s="15" t="str">
-        <x:v>Blank/oversize input, public/internal visibility and encoded notes checked through the portal contract. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P13/P14/P15 persist author/time and visibility, reject blank notes and append corrections while retaining earlier entries. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD12" s="15" t="str">
-        <x:v>General notes need persisted author/time and correction history.</x:v>
+        <x:v>Corrections are appended; there is no destructive note-edit endpoint.</x:v>
       </x:c>
       <x:c r="AE12" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="95.0999984741211" customHeight="1">
@@ -3028,10 +3028,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AC13" s="15" t="str">
-        <x:v>M3 lifecycle saves resolution summary/actor/time and rejects unauthorised or invalid closure. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P24/P25 and M3 E01/E02 verify required feedback/resolution summary, actor/time and legal authorised closure. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD13" s="15" t="str">
-        <x:v>Real-account portal acceptance remains separate from the verified status API.</x:v>
+        <x:v>No automatic closure or reopening was committed.</x:v>
       </x:c>
       <x:c r="AE13" s="15" t="str">
         <x:v>Verified</x:v>
@@ -3109,34 +3109,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W14" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X14" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y14" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z14" s="17" t="n">
         <x:f>IF(X14="Met",1,IF(X14="Partially Met",0.5,IF(X14="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA14" s="17" t="n">
         <x:f>IF(Y14="Met",1,IF(Y14="Partially Met",0.5,IF(Y14="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB14" s="17" t="n">
         <x:f>IF(COUNT(Z14:AA14)=2,SUM(Z14:AA14),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC14" s="15" t="str">
-        <x:v>Bianca’s known-data calculator and management controller/zero counts are exercised. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>SM01–SM12 and P21/P27 verify lifecycle/overdue calculations, saved changes, zero counts and requester reporting denial. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD14" s="15" t="str">
-        <x:v>Saved management data and refresh against persistent changes await integration.</x:v>
+        <x:v>Summary reads are unpaginated and the full pilot response-time criterion remains separate.</x:v>
       </x:c>
       <x:c r="AE14" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="95.0999984741211" customHeight="1">
@@ -3211,34 +3211,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W15" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X15" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y15" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z15" s="17" t="n">
         <x:f>IF(X15="Met",1,IF(X15="Partially Met",0.5,IF(X15="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA15" s="17" t="n">
         <x:f>IF(Y15="Met",1,IF(Y15="Partially Met",0.5,IF(Y15="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB15" s="17" t="n">
         <x:f>IF(COUNT(Z15:AA15)=2,SUM(Z15:AA15),"Pending")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC15" s="15" t="str">
-        <x:v>Management category/status selections filter synthetic reporting data and counts. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P21/P27 and the management UI checks verify saved matching references, category/status selection, clear selections and zero-match feedback. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD15" s="15" t="str">
-        <x:v>The persisted management overview and individual matching request presentation remain incomplete.</x:v>
+        <x:v>Management sees request reference/category/status rather than requester private details.</x:v>
       </x:c>
       <x:c r="AE15" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="95.0999984741211" customHeight="1">
@@ -3317,34 +3317,34 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="W16" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X16" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y16" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z16" s="17" t="n">
         <x:f>IF(X16="Met",1,IF(X16="Partially Met",0.5,IF(X16="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA16" s="17" t="n">
         <x:f>IF(Y16="Met",1,IF(Y16="Partially Met",0.5,IF(Y16="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB16" s="17" t="n">
         <x:f>IF(COUNT(Z16:AA16)=2,SUM(Z16:AA16),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC16" s="15" t="str">
-        <x:v>Status history is transactional and persisted with actor/time. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P18/P28 and recovery.json verify creation, ownership, status, scheduling and note audit with actor/time, restart survival and exact restore. Ordinary users have no audit-edit endpoint. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD16" s="15" t="str">
-        <x:v>Creation/ownership/priority/due-date/note audit, restart and immutability coverage remain incomplete.</x:v>
+        <x:v>Database administrators can alter tables; application append-only behaviour is not tamper-proof external archival.</x:v>
       </x:c>
       <x:c r="AE16" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="95.0999984741211" customHeight="1">
@@ -3423,17 +3423,17 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="W17" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X17" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y17" s="15" t="str">
         <x:v>Met</x:v>
       </x:c>
       <x:c r="Z17" s="17" t="n">
         <x:f>IF(X17="Met",1,IF(X17="Partially Met",0.5,IF(X17="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA17" s="17" t="n">
         <x:f>IF(Y17="Met",1,IF(Y17="Partially Met",0.5,IF(Y17="Not Met",0,"Pending")))</x:f>
@@ -3441,16 +3441,16 @@
       </x:c>
       <x:c r="AB17" s="17" t="n">
         <x:f>IF(COUNT(Z17:AA17)=2,SUM(Z17:AA17),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC17" s="15" t="str">
-        <x:v>Sign-in/session controller, role injection denial, signed-out access and permission refresh checked. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P01/P02/P29 use real password hashes, server-owned roles and stored-account revocation; UI/M3 cases deny signed-out and ambiguous principals. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD17" s="15" t="str">
-        <x:v>There is no registered real account adapter or verified enabled-account credential store.</x:v>
+        <x:v>No public self-registration, password reset, MFA or login rate limiting is delivered; these remain production security limitations.</x:v>
       </x:c>
       <x:c r="AE17" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="95.0999984741211" customHeight="1">
@@ -3525,34 +3525,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W18" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X18" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y18" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z18" s="17" t="n">
         <x:f>IF(X18="Met",1,IF(X18="Partially Met",0.5,IF(X18="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA18" s="17" t="n">
         <x:f>IF(Y18="Met",1,IF(Y18="Partially Met",0.5,IF(Y18="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB18" s="17" t="n">
         <x:f>IF(COUNT(Z18:AA18)=2,SUM(Z18:AA18),"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC18" s="15" t="str">
-        <x:v>Controlled priority input and protected update form call a versioned store contract. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P05/P16/P17/P20 verify default Normal, saved changes, filtering, numeric priority sorting and invalid/requester denial. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD18" s="15" t="str">
-        <x:v>Default and updated priorities must be persisted and used by real sorting/filtering.</x:v>
+        <x:v>Priority is one of Low, Normal or High; no custom priority editor is provided.</x:v>
       </x:c>
       <x:c r="AE18" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="95.0999984741211" customHeight="1">
@@ -3627,34 +3627,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W19" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X19" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y19" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z19" s="17" t="n">
         <x:f>IF(X19="Met",1,IF(X19="Partially Met",0.5,IF(X19="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA19" s="17" t="n">
         <x:f>IF(Y19="Met",1,IF(Y19="Partially Met",0.5,IF(Y19="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB19" s="17" t="n">
         <x:f>IF(COUNT(Z19:AA19)=2,SUM(Z19:AA19),"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC19" s="15" t="str">
-        <x:v>UTC due-date binding and Bianca’s open/overdue/null-date boundaries checked. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P16/P17/P18/P21 verify valid UTC due dates, audit, malformed-date rejection and overdue rules; SM checks cover null and terminal dates. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD19" s="15" t="str">
-        <x:v>Saved due-date audit and actual overdue records await Michael’s adapter.</x:v>
+        <x:v>Forms state UTC explicitly; user-local timezone preferences are not provided.</x:v>
       </x:c>
       <x:c r="AE19" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="95.0999984741211" customHeight="1">
@@ -3754,10 +3754,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AC20" s="15" t="str">
-        <x:v>Existing read/status access matrix passes; new role/category, privacy and session checks pass. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>Read, API, UI and persistent role/ownership/category cases pass without an unauthorised disclosure or mutation in the tested set. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD20" s="15" t="str">
-        <x:v>Confidence is limited to tested surfaces; review every new adapter/query before final acceptance.</x:v>
+        <x:v>This is the defined access-test set, not an external penetration assessment.</x:v>
       </x:c>
       <x:c r="AE20" s="15" t="str">
         <x:v>Verified</x:v>
@@ -3841,7 +3841,7 @@
         <x:v>239</x:v>
       </x:c>
       <x:c r="W21" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>NOT IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X21" s="15" t="str">
         <x:v>Not Met</x:v>
@@ -3862,10 +3862,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="AC21" s="15" t="str">
-        <x:v>PR20 records a paced database-read exercise; original user-visible workload is not established. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>Michael’s existing paced database-read measurement remains available; correctness journeys now exercise all real portal adapters. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD21" s="15" t="str">
-        <x:v>Four separate user-visible operations, specified dataset/load, failures and cold start remain unverified.</x:v>
+        <x:v>The specified 10-user, 1,000-request, four-operation browser workload, separate visible-result timings and cold start were not executed. Not delivered.</x:v>
       </x:c>
       <x:c r="AE21" s="15" t="str">
         <x:v>Not delivered</x:v>
@@ -3947,34 +3947,34 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="W22" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X22" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y22" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z22" s="17" t="n">
         <x:f>IF(X22="Met",1,IF(X22="Partially Met",0.5,IF(X22="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA22" s="17" t="n">
         <x:f>IF(Y22="Met",1,IF(Y22="Partially Met",0.5,IF(Y22="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB22" s="17" t="n">
         <x:f>IF(COUNT(Z22:AA22)=2,SUM(Z22:AA22),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC22" s="15" t="str">
-        <x:v>PostgreSQL status rollback/concurrency verified; submission keys are preserved by the UI contract. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P04a/P06/P11a/P12/P23/P28 and the database suite verify submission/assignment/status rollback, competing claims, durable idempotency and application restart. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD22" s="15" t="str">
-        <x:v>Durable idempotency, assignment atomicity and full restart acceptance remain open.</x:v>
+        <x:v>Controlled local PostgreSQL; infrastructure failover was not tested.</x:v>
       </x:c>
       <x:c r="AE22" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="95.0999984741211" customHeight="1">
@@ -4049,13 +4049,13 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W23" s="15" t="str">
-        <x:v>NOT IMPLEMENTED</x:v>
+        <x:v>PARTIALLY IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X23" s="15" t="str">
         <x:v>Not Met</x:v>
       </x:c>
       <x:c r="Y23" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z23" s="17" t="n">
         <x:f>IF(X23="Met",1,IF(X23="Partially Met",0.5,IF(X23="Not Met",0,"Pending")))</x:f>
@@ -4063,17 +4063,17 @@
       </x:c>
       <x:c r="AA23" s="17" t="n">
         <x:f>IF(Y23="Met",1,IF(Y23="Partially Met",0.5,IF(Y23="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB23" s="17" t="n">
         <x:f>IF(COUNT(Z23:AA23)=2,SUM(Z23:AA23),"Pending")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AC23" s="15" t="str">
-        <x:v>No representative participant exercise is supplied. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>Cameron observed all five participants following the same task: 3/5 reported completion within 300 seconds without coaching. Times, errors and coaching recorded. docs/evidence/m4-final-20261018/usability.md</x:v>
       </x:c>
       <x:c r="AD23" s="15" t="str">
-        <x:v>Five-participant task/time/error records are required; synthetic UI checks are not usability acceptance.</x:v>
+        <x:v>Four-of-five uncoached threshold failed. P2/P3 chose a different category; strict task-conforming uncoached completion is 2/5. Small local convenience sample.</x:v>
       </x:c>
       <x:c r="AE23" s="15" t="str">
         <x:v>Not delivered</x:v>
@@ -4154,14 +4154,14 @@
         <x:v>PARTIALLY IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X24" s="15" t="str">
-        <x:v>Not Met</x:v>
+        <x:v>Partially Met</x:v>
       </x:c>
       <x:c r="Y24" s="15" t="str">
         <x:v>Partially Met</x:v>
       </x:c>
       <x:c r="Z24" s="17" t="n">
         <x:f>IF(X24="Met",1,IF(X24="Partially Met",0.5,IF(X24="Not Met",0,"Pending")))</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="AA24" s="17" t="n">
         <x:f>IF(Y24="Met",1,IF(Y24="Partially Met",0.5,IF(Y24="Not Met",0,"Pending")))</x:f>
@@ -4169,13 +4169,13 @@
       </x:c>
       <x:c r="AB24" s="17" t="n">
         <x:f>IF(COUNT(Z24:AA24)=2,SUM(Z24:AA24),"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AC24" s="15" t="str">
-        <x:v>Current 558px browser layout inspected; keyboard sign-in and submission exercised. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>Chrome sign-in layouts at 360/1366 show no horizontal overflow. Keyboard sign-in, category selection, text entry, visible focus and submission were exercised in the in-app browser. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD24" s="15" t="str">
-        <x:v>360/1366 Chrome-and-Edge matrix and complete keyboard/error journey remain unverified.</x:v>
+        <x:v>The complete Chrome/Edge screen matrix and keyboard validation-error journey are not yet evidenced.</x:v>
       </x:c>
       <x:c r="AE24" s="15" t="str">
         <x:v>Not delivered</x:v>
@@ -4278,10 +4278,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AC25" s="15" t="str">
-        <x:v>M3 HTTPS test host and PR20 local HTTPS redirect evidence exist; Secure cookies retained. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>Persistent tests use HTTPS with a pinned generated certificate; normal application cookies and antiforgery cookies require HTTPS. Michael’s redirect evidence is retained. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD25" s="15" t="str">
-        <x:v>Final deployed certificate, sign-in/protected browser pages and mixed-content checks remain unverified.</x:v>
+        <x:v>No public host or browser-trusted deployed certificate exists. The isolated participant preview uses loopback HTTP with synthetic accounts; it does not satisfy deployed HTTPS acceptance.</x:v>
       </x:c>
       <x:c r="AE25" s="15" t="str">
         <x:v>Not delivered</x:v>
@@ -4359,34 +4359,34 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="W26" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X26" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y26" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z26" s="17" t="n">
         <x:f>IF(X26="Met",1,IF(X26="Partially Met",0.5,IF(X26="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA26" s="17" t="n">
         <x:f>IF(Y26="Met",1,IF(Y26="Partially Met",0.5,IF(Y26="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB26" s="17" t="n">
         <x:f>IF(COUNT(Z26:AA26)=2,SUM(Z26:AA26),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC26" s="15" t="str">
-        <x:v>Michael’s PR20 restores tables and matching record counts to a separate database. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>recovery.json records a fresh backup, 0.917-second conservative age and 0.676-second restore/verification. Request, eligible owner, five status-history rows, six notes and scheduling audit match exactly. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD26" s="15" t="str">
-        <x:v>Backup age, timed restoration, RPO/RTO and consistent owner/history recovery are not established.</x:v>
+        <x:v>Small synthetic local dataset and manual backup. Automatic scheduling, off-site retention and hosted disaster recovery are not established.</x:v>
       </x:c>
       <x:c r="AE26" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="95.0999984741211" customHeight="1">
@@ -4465,34 +4465,34 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="W27" s="15" t="str">
-        <x:v>PARTIALLY IMPLEMENTED</x:v>
+        <x:v>IMPLEMENTED</x:v>
       </x:c>
       <x:c r="X27" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Y27" s="15" t="str">
-        <x:v>Partially Met</x:v>
+        <x:v>Met</x:v>
       </x:c>
       <x:c r="Z27" s="17" t="n">
         <x:f>IF(X27="Met",1,IF(X27="Partially Met",0.5,IF(X27="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA27" s="17" t="n">
         <x:f>IF(Y27="Met",1,IF(Y27="Partially Met",0.5,IF(Y27="Not Met",0,"Pending")))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB27" s="17" t="n">
         <x:f>IF(COUNT(Z27:AA27)=2,SUM(Z27:AA27),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AC27" s="15" t="str">
-        <x:v>M3 safe-error checks and new action-specific messages exclude private payloads from responses. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>P23 and existing safe-error cases check dummy-secret/private-content non-disclosure; P04a/P11a/P23 verify action-specific failure titles. Custom logs record exception type only. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD27" s="15" t="str">
-        <x:v>A complete dummy-secret/private-content log audit remains outstanding.</x:v>
+        <x:v>Sensitive-data logging must remain disabled when deploying or changing providers.</x:v>
       </x:c>
       <x:c r="AE27" s="15" t="str">
-        <x:v>Not delivered</x:v>
+        <x:v>Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="95.0999984741211" customHeight="1">
@@ -4598,10 +4598,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AC28" s="15" t="str">
-        <x:v>Submission/access/assignment/status/reporting rules accept controlled test inputs; repeatable suites and negative controls exist. Evidence: docs/testing-m3.md; docs/evidence/m4-cameron-20261018/summary.md; PR20 where relevant.</x:v>
+        <x:v>Pure lifecycle/ownership/summary checks, fixture UI checks and repeatable real-adapter scenarios run independently of production data; illegal transitions and injected faults are detected. docs/evidence/m4-final-20261018/summary.md</x:v>
       </x:c>
       <x:c r="AD28" s="15" t="str">
-        <x:v>Testability does not imply that the corresponding persistent product journeys are delivered.</x:v>
+        <x:v>Custom executable harnesses require explicit CI invocation rather than standard test discovery.</x:v>
       </x:c>
       <x:c r="AE28" s="15" t="str">
         <x:v>Verified</x:v>
@@ -4755,9 +4755,9 @@
       <x:c r="K38" s="4"/>
       <x:c r="L38" s="4"/>
     </x:row>
-    <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="40" ht="14.25" hidden="0" customHeight="1">
       <x:c r="W40" s="16" t="str">
-        <x:v>M4 checkpoint, not frozen final acceptance</x:v>
+        <x:v>M4 final assessment</x:v>
       </x:c>
       <x:c r="X40" s="16"/>
     </x:row>
@@ -4767,7 +4767,7 @@
       </x:c>
       <x:c r="X41" s="22" t="n">
         <x:f>IF(COUNT(Z2:AA28)=COUNTA(Requirements!D2:E28),SUM(Z2:AA28)/COUNTA(Requirements!D2:E28),"Pending")</x:f>
-        <x:v>0.4722222222222222</x:v>
+        <x:v>0.8981481481481481</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="14.25" hidden="0" customHeight="1">
@@ -4784,7 +4784,7 @@
       </x:c>
       <x:c r="X43" s="15" t="n">
         <x:f>SUM(Z2:AA28)</x:f>
-        <x:v>25.5</x:v>
+        <x:v>48.5</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="14.25" hidden="0" customHeight="1">
@@ -4801,7 +4801,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="X45" s="15" t="str">
-        <x:v>Provisional; team adapters and final release still pending</x:v>
+        <x:v>Controlled staging; actual participant results only; no production approval</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -4809,7 +4809,7 @@
         <x:v>Scoring</x:v>
       </x:c>
       <x:c r="X46" s="15" t="str">
-        <x:v>Met 1; Partially Met 0.5; Not Met 0. No approved baseline removals.</x:v>
+        <x:v>Met 1; Partially Met 0.5; Not Met 0. Original 54 criteria retained.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>